<commit_message>
feat: improve task overdue detection and UI representation
- Refactored overdue detection logic to utilize a new `getTaskOverdueState` function for better clarity and maintainability.
- Updated task list view to visually indicate overdue tasks based on specific fields (endDate, uatDate, prdDate).
- Enhanced utility functions to streamline overdue checks and improve task management efficiency.
- Updated taskDB.xlsx with new data reflecting changes in task management.
</commit_message>
<xml_diff>
--- a/data/taskDB.xlsx
+++ b/data/taskDB.xlsx
@@ -804,7 +804,7 @@
         <v>2026-09-01T07:23:24.979Z</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-09-04T12:51:27.047Z</v>
+        <v>2026-09-07T03:06:35.964Z</v>
       </c>
     </row>
     <row r="3">
@@ -824,7 +824,7 @@
         <v>2026-09-01T07:23:24.981Z</v>
       </c>
       <c r="F3" t="str">
-        <v>2026-09-04T12:51:27.053Z</v>
+        <v>2026-09-07T03:06:35.994Z</v>
       </c>
     </row>
     <row r="4">
@@ -844,7 +844,7 @@
         <v>2026-09-01T07:23:24.983Z</v>
       </c>
       <c r="F4" t="str">
-        <v>2026-09-04T12:51:27.066Z</v>
+        <v>2026-09-07T03:06:36.036Z</v>
       </c>
     </row>
     <row r="5">
@@ -864,7 +864,7 @@
         <v>2026-09-01T07:23:24.985Z</v>
       </c>
       <c r="F5" t="str">
-        <v>2026-09-04T12:51:27.059Z</v>
+        <v>2026-09-07T03:06:36.011Z</v>
       </c>
     </row>
     <row r="6">
@@ -884,7 +884,7 @@
         <v>2026-09-01T07:23:24.988Z</v>
       </c>
       <c r="F6" t="str">
-        <v>2026-09-04T12:51:27.071Z</v>
+        <v>2026-09-07T03:06:36.058Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: refactor task creation and management UI components
- Updated task creation logic to utilize a default status ID for new tasks.
- Refactored inline task creation component to simplify state management and remove unnecessary props.
- Enhanced Kanban view by removing inline task creation and streamlining task display.
- Adjusted task form dialog to reset state upon closing, improving user experience.
- Updated taskDB.xlsx to reflect changes in task management structure.
</commit_message>
<xml_diff>
--- a/data/taskDB.xlsx
+++ b/data/taskDB.xlsx
@@ -804,7 +804,7 @@
         <v>2026-09-01T07:23:24.979Z</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-09-07T03:06:35.964Z</v>
+        <v>2026-09-07T04:07:14.587Z</v>
       </c>
     </row>
     <row r="3">
@@ -824,7 +824,7 @@
         <v>2026-09-01T07:23:24.981Z</v>
       </c>
       <c r="F3" t="str">
-        <v>2026-09-07T03:06:35.994Z</v>
+        <v>2026-09-07T04:07:14.596Z</v>
       </c>
     </row>
     <row r="4">
@@ -844,7 +844,7 @@
         <v>2026-09-01T07:23:24.983Z</v>
       </c>
       <c r="F4" t="str">
-        <v>2026-09-07T03:06:36.036Z</v>
+        <v>2026-09-07T04:07:14.611Z</v>
       </c>
     </row>
     <row r="5">
@@ -864,7 +864,7 @@
         <v>2026-09-01T07:23:24.985Z</v>
       </c>
       <c r="F5" t="str">
-        <v>2026-09-07T03:06:36.011Z</v>
+        <v>2026-09-07T04:07:14.603Z</v>
       </c>
     </row>
     <row r="6">
@@ -884,7 +884,7 @@
         <v>2026-09-01T07:23:24.988Z</v>
       </c>
       <c r="F6" t="str">
-        <v>2026-09-07T03:06:36.058Z</v>
+        <v>2026-09-07T04:07:14.619Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: enhance task and team member management with owner support
- Updated task model to include an owner field, allowing for better task ownership tracking.
- Modified team member model to add new fields: name, email, and employeeId for improved member details.
- Enhanced task forms and dialogs to support owner selection and display.
- Updated API endpoints to handle owner assignments during task creation and updates.
- Refactored UI components to display task owners effectively across the application.
- Updated taskDB.xlsx and related repositories to reflect changes in task and team member structures.
</commit_message>
<xml_diff>
--- a/data/taskDB.xlsx
+++ b/data/taskDB.xlsx
@@ -436,13 +436,13 @@
         <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
       </c>
       <c r="B2" t="str">
-        <v>FWF Task Manager</v>
+        <v>FWF Task</v>
       </c>
       <c r="C2" t="str">
         <v>Foreigner Worker Fund</v>
       </c>
       <c r="D2" t="str">
-        <v>#1E3A5F</v>
+        <v>#3B82F6</v>
       </c>
       <c r="E2" t="str">
         <v>0</v>
@@ -451,7 +451,7 @@
         <v>2026-09-01T07:23:24.969Z</v>
       </c>
       <c r="G2" t="str">
-        <v>2026-09-01T07:23:24.969Z</v>
+        <v>2026-09-08T07:06:14.659Z</v>
       </c>
     </row>
   </sheetData>
@@ -804,7 +804,7 @@
         <v>2026-09-01T07:23:24.979Z</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-09-07T04:07:14.587Z</v>
+        <v>2026-09-08T07:44:34.904Z</v>
       </c>
     </row>
     <row r="3">
@@ -824,7 +824,7 @@
         <v>2026-09-01T07:23:24.981Z</v>
       </c>
       <c r="F3" t="str">
-        <v>2026-09-07T04:07:14.596Z</v>
+        <v>2026-09-08T07:44:34.911Z</v>
       </c>
     </row>
     <row r="4">
@@ -844,7 +844,7 @@
         <v>2026-09-01T07:23:24.983Z</v>
       </c>
       <c r="F4" t="str">
-        <v>2026-09-07T04:07:14.611Z</v>
+        <v>2026-09-08T07:44:34.925Z</v>
       </c>
     </row>
     <row r="5">
@@ -864,7 +864,7 @@
         <v>2026-09-01T07:23:24.985Z</v>
       </c>
       <c r="F5" t="str">
-        <v>2026-09-07T04:07:14.603Z</v>
+        <v>2026-09-08T07:44:34.917Z</v>
       </c>
     </row>
     <row r="6">
@@ -884,7 +884,7 @@
         <v>2026-09-01T07:23:24.988Z</v>
       </c>
       <c r="F6" t="str">
-        <v>2026-09-07T04:07:14.619Z</v>
+        <v>2026-09-08T07:44:34.932Z</v>
       </c>
     </row>
   </sheetData>
@@ -896,28 +896,37 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:J9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>id</v>
       </c>
       <c r="B1" t="str">
+        <v>name</v>
+      </c>
+      <c r="C1" t="str">
         <v>nickname</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
+        <v>email</v>
+      </c>
+      <c r="E1" t="str">
+        <v>employeeId</v>
+      </c>
+      <c r="F1" t="str">
         <v>color</v>
       </c>
-      <c r="D1" t="str">
+      <c r="G1" t="str">
         <v>isActive</v>
       </c>
-      <c r="E1" t="str">
+      <c r="H1" t="str">
         <v>sortOrder</v>
       </c>
-      <c r="F1" t="str">
+      <c r="I1" t="str">
         <v>createdAt</v>
       </c>
-      <c r="G1" t="str">
+      <c r="J1" t="str">
         <v>updatedAt</v>
       </c>
     </row>
@@ -926,22 +935,31 @@
         <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
       </c>
       <c r="B2" t="str">
+        <v>Natchanon Srichom</v>
+      </c>
+      <c r="C2" t="str">
         <v>Guny</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
+        <v>g.ncs0925@gmail.com</v>
+      </c>
+      <c r="E2" t="str">
+        <v>65357</v>
+      </c>
+      <c r="F2" t="str">
         <v>#22C55E</v>
       </c>
-      <c r="D2" t="str">
+      <c r="G2" t="str">
         <v>TRUE</v>
       </c>
-      <c r="E2" t="str">
-        <v>0</v>
-      </c>
-      <c r="F2" t="str">
+      <c r="H2" t="str">
+        <v>0</v>
+      </c>
+      <c r="I2" t="str">
         <v>2026-09-01T07:26:41.854Z</v>
       </c>
-      <c r="G2" t="str">
-        <v>2026-09-04T11:53:20.413Z</v>
+      <c r="J2" t="str">
+        <v>2026-09-08T07:18:05.956Z</v>
       </c>
     </row>
     <row r="3">
@@ -949,21 +967,30 @@
         <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
       </c>
       <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
         <v>Cream</v>
       </c>
-      <c r="C3" t="str">
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
         <v>#EF4444</v>
       </c>
-      <c r="D3" t="str">
+      <c r="G3" t="str">
         <v>TRUE</v>
       </c>
-      <c r="E3" t="str">
+      <c r="H3" t="str">
         <v>1</v>
       </c>
-      <c r="F3" t="str">
+      <c r="I3" t="str">
         <v>2026-09-04T08:31:09.214Z</v>
       </c>
-      <c r="G3" t="str">
+      <c r="J3" t="str">
         <v>2026-09-04T11:53:27.762Z</v>
       </c>
     </row>
@@ -972,21 +999,30 @@
         <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
       </c>
       <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
         <v>P Aek</v>
       </c>
-      <c r="C4" t="str">
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
         <v>#F97316</v>
       </c>
-      <c r="D4" t="str">
+      <c r="G4" t="str">
         <v>TRUE</v>
       </c>
-      <c r="E4" t="str">
+      <c r="H4" t="str">
         <v>2</v>
       </c>
-      <c r="F4" t="str">
+      <c r="I4" t="str">
         <v>2026-09-04T08:31:15.973Z</v>
       </c>
-      <c r="G4" t="str">
+      <c r="J4" t="str">
         <v>2026-09-04T11:53:35.476Z</v>
       </c>
     </row>
@@ -995,21 +1031,30 @@
         <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
       </c>
       <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
         <v>P Juu</v>
       </c>
-      <c r="C5" t="str">
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
         <v>#3B82F6</v>
       </c>
-      <c r="D5" t="str">
+      <c r="G5" t="str">
         <v>TRUE</v>
       </c>
-      <c r="E5" t="str">
+      <c r="H5" t="str">
         <v>3</v>
       </c>
-      <c r="F5" t="str">
+      <c r="I5" t="str">
         <v>2026-09-04T08:31:24.760Z</v>
       </c>
-      <c r="G5" t="str">
+      <c r="J5" t="str">
         <v>2026-09-04T11:53:44.607Z</v>
       </c>
     </row>
@@ -1018,21 +1063,30 @@
         <v>55d6e756-c40c-4755-84ab-c3458437acd6</v>
       </c>
       <c r="B6" t="str">
+        <v/>
+      </c>
+      <c r="C6" t="str">
         <v>Frame</v>
       </c>
-      <c r="C6" t="str">
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
         <v>#8B5CF6</v>
       </c>
-      <c r="D6" t="str">
+      <c r="G6" t="str">
         <v>TRUE</v>
       </c>
-      <c r="E6" t="str">
+      <c r="H6" t="str">
         <v>4</v>
       </c>
-      <c r="F6" t="str">
+      <c r="I6" t="str">
         <v>2026-09-04T08:31:29.670Z</v>
       </c>
-      <c r="G6" t="str">
+      <c r="J6" t="str">
         <v>2026-09-04T11:53:59.480Z</v>
       </c>
     </row>
@@ -1041,21 +1095,30 @@
         <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
       </c>
       <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
         <v>Mild</v>
       </c>
-      <c r="C7" t="str">
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
         <v>#EC4899</v>
       </c>
-      <c r="D7" t="str">
+      <c r="G7" t="str">
         <v>TRUE</v>
       </c>
-      <c r="E7" t="str">
+      <c r="H7" t="str">
         <v>5</v>
       </c>
-      <c r="F7" t="str">
+      <c r="I7" t="str">
         <v>2026-09-04T08:31:33.588Z</v>
       </c>
-      <c r="G7" t="str">
+      <c r="J7" t="str">
         <v>2026-09-04T11:54:13.639Z</v>
       </c>
     </row>
@@ -1064,21 +1127,30 @@
         <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
       <c r="B8" t="str">
+        <v/>
+      </c>
+      <c r="C8" t="str">
         <v>Breez</v>
       </c>
-      <c r="C8" t="str">
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8" t="str">
         <v>#75D7F0</v>
       </c>
-      <c r="D8" t="str">
+      <c r="G8" t="str">
         <v>TRUE</v>
       </c>
-      <c r="E8" t="str">
+      <c r="H8" t="str">
         <v>6</v>
       </c>
-      <c r="F8" t="str">
+      <c r="I8" t="str">
         <v>2026-09-04T08:31:52.262Z</v>
       </c>
-      <c r="G8" t="str">
+      <c r="J8" t="str">
         <v>2026-09-04T11:54:20.446Z</v>
       </c>
     </row>
@@ -1087,34 +1159,43 @@
         <v>190c2d73-d236-4277-a3e1-b6004555ac94</v>
       </c>
       <c r="B9" t="str">
+        <v/>
+      </c>
+      <c r="C9" t="str">
         <v>Prink</v>
       </c>
-      <c r="C9" t="str">
+      <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
         <v>#F0EC75</v>
       </c>
-      <c r="D9" t="str">
+      <c r="G9" t="str">
         <v>TRUE</v>
       </c>
-      <c r="E9" t="str">
+      <c r="H9" t="str">
         <v>7</v>
       </c>
-      <c r="F9" t="str">
+      <c r="I9" t="str">
         <v>2026-09-04T08:32:04.538Z</v>
       </c>
-      <c r="G9" t="str">
+      <c r="J9" t="str">
         <v>2026-09-04T11:54:26.641Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J9"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P19"/>
+  <dimension ref="A1:Q21"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1160,9 +1241,12 @@
         <v>assigneeId</v>
       </c>
       <c r="O1" t="str">
+        <v>ownerId</v>
+      </c>
+      <c r="P1" t="str">
         <v>createdAt</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
         <v>updatedAt</v>
       </c>
     </row>
@@ -1210,9 +1294,12 @@
         <v>55d6e756-c40c-4755-84ab-c3458437acd6</v>
       </c>
       <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
         <v>2026-09-04T09:22:21.943Z</v>
       </c>
-      <c r="P2" t="str">
+      <c r="Q2" t="str">
         <v>2026-09-04T12:29:28.753Z</v>
       </c>
     </row>
@@ -1260,9 +1347,12 @@
         <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
       </c>
       <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
         <v>2026-09-04T09:24:04.693Z</v>
       </c>
-      <c r="P3" t="str">
+      <c r="Q3" t="str">
         <v>2026-09-04T12:29:22.917Z</v>
       </c>
     </row>
@@ -1310,9 +1400,12 @@
         <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
       </c>
       <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
         <v>2026-09-04T09:24:33.365Z</v>
       </c>
-      <c r="P4" t="str">
+      <c r="Q4" t="str">
         <v>2026-09-04T12:29:18.513Z</v>
       </c>
     </row>
@@ -1360,9 +1453,12 @@
         <v>55d6e756-c40c-4755-84ab-c3458437acd6</v>
       </c>
       <c r="O5" t="str">
+        <v/>
+      </c>
+      <c r="P5" t="str">
         <v>2026-09-04T09:25:10.002Z</v>
       </c>
-      <c r="P5" t="str">
+      <c r="Q5" t="str">
         <v>2026-09-04T12:29:13.377Z</v>
       </c>
     </row>
@@ -1410,9 +1506,12 @@
         <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
       </c>
       <c r="O6" t="str">
+        <v/>
+      </c>
+      <c r="P6" t="str">
         <v>2026-09-04T09:26:00.676Z</v>
       </c>
-      <c r="P6" t="str">
+      <c r="Q6" t="str">
         <v>2026-09-04T12:29:08.647Z</v>
       </c>
     </row>
@@ -1460,9 +1559,12 @@
         <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
       </c>
       <c r="O7" t="str">
+        <v/>
+      </c>
+      <c r="P7" t="str">
         <v>2026-09-04T09:27:00.612Z</v>
       </c>
-      <c r="P7" t="str">
+      <c r="Q7" t="str">
         <v>2026-09-04T11:32:30.909Z</v>
       </c>
     </row>
@@ -1510,9 +1612,12 @@
         <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
       <c r="O8" t="str">
+        <v/>
+      </c>
+      <c r="P8" t="str">
         <v>2026-09-04T09:29:47.993Z</v>
       </c>
-      <c r="P8" t="str">
+      <c r="Q8" t="str">
         <v>2026-09-04T09:41:39.538Z</v>
       </c>
     </row>
@@ -1560,9 +1665,12 @@
         <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
       </c>
       <c r="O9" t="str">
+        <v/>
+      </c>
+      <c r="P9" t="str">
         <v>2026-09-04T09:32:18.156Z</v>
       </c>
-      <c r="P9" t="str">
+      <c r="Q9" t="str">
         <v>2026-09-04T12:29:03.482Z</v>
       </c>
     </row>
@@ -1610,9 +1718,12 @@
         <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
       </c>
       <c r="O10" t="str">
+        <v/>
+      </c>
+      <c r="P10" t="str">
         <v>2026-09-04T09:33:03.132Z</v>
       </c>
-      <c r="P10" t="str">
+      <c r="Q10" t="str">
         <v>2026-09-04T11:32:35.144Z</v>
       </c>
     </row>
@@ -1660,9 +1771,12 @@
         <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
       <c r="O11" t="str">
+        <v/>
+      </c>
+      <c r="P11" t="str">
         <v>2026-09-04T09:33:38.656Z</v>
       </c>
-      <c r="P11" t="str">
+      <c r="Q11" t="str">
         <v>2026-09-04T09:41:08.425Z</v>
       </c>
     </row>
@@ -1704,16 +1818,19 @@
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
       <c r="M12" t="str">
-        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+        <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
       </c>
       <c r="N12" t="str">
-        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
+        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
       </c>
       <c r="O12" t="str">
+        <v/>
+      </c>
+      <c r="P12" t="str">
         <v>2026-09-04T09:34:04.072Z</v>
       </c>
-      <c r="P12" t="str">
-        <v>2026-09-04T09:40:35.751Z</v>
+      <c r="Q12" t="str">
+        <v>2026-09-08T07:00:11.973Z</v>
       </c>
     </row>
     <row r="13">
@@ -1754,16 +1871,19 @@
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
       <c r="M13" t="str">
-        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
       </c>
       <c r="N13" t="str">
         <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
       </c>
       <c r="O13" t="str">
+        <v/>
+      </c>
+      <c r="P13" t="str">
         <v>2026-09-04T09:43:36.886Z</v>
       </c>
-      <c r="P13" t="str">
-        <v>2026-09-04T09:45:31.790Z</v>
+      <c r="Q13" t="str">
+        <v>2026-09-08T03:13:32.587Z</v>
       </c>
     </row>
     <row r="14">
@@ -1804,16 +1924,19 @@
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
       <c r="M14" t="str">
-        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
       </c>
       <c r="N14" t="str">
         <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
       </c>
       <c r="O14" t="str">
+        <v/>
+      </c>
+      <c r="P14" t="str">
         <v>2026-09-04T09:43:56.520Z</v>
       </c>
-      <c r="P14" t="str">
-        <v>2026-09-04T09:45:22.510Z</v>
+      <c r="Q14" t="str">
+        <v>2026-09-08T03:12:47.743Z</v>
       </c>
     </row>
     <row r="15">
@@ -1854,16 +1977,19 @@
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
       <c r="M15" t="str">
-        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
       </c>
       <c r="N15" t="str">
-        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
+        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
       </c>
       <c r="O15" t="str">
+        <v/>
+      </c>
+      <c r="P15" t="str">
         <v>2026-09-04T09:44:42.509Z</v>
       </c>
-      <c r="P15" t="str">
-        <v>2026-09-04T09:44:49.331Z</v>
+      <c r="Q15" t="str">
+        <v>2026-09-08T07:00:38.382Z</v>
       </c>
     </row>
     <row r="16">
@@ -1910,9 +2036,12 @@
         <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
       </c>
       <c r="O16" t="str">
+        <v/>
+      </c>
+      <c r="P16" t="str">
         <v>2026-09-04T09:47:39.827Z</v>
       </c>
-      <c r="P16" t="str">
+      <c r="Q16" t="str">
         <v>2026-09-04T09:47:39.843Z</v>
       </c>
     </row>
@@ -1960,9 +2089,12 @@
         <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
       </c>
       <c r="O17" t="str">
+        <v/>
+      </c>
+      <c r="P17" t="str">
         <v>2026-09-04T09:48:58.057Z</v>
       </c>
-      <c r="P17" t="str">
+      <c r="Q17" t="str">
         <v>2026-09-04T09:48:58.073Z</v>
       </c>
     </row>
@@ -2010,9 +2142,12 @@
         <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
       </c>
       <c r="O18" t="str">
+        <v/>
+      </c>
+      <c r="P18" t="str">
         <v>2026-09-04T09:50:04.917Z</v>
       </c>
-      <c r="P18" t="str">
+      <c r="Q18" t="str">
         <v>2026-09-04T10:15:31.436Z</v>
       </c>
     </row>
@@ -2060,22 +2195,131 @@
         <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
       </c>
       <c r="O19" t="str">
+        <v/>
+      </c>
+      <c r="P19" t="str">
         <v>2026-09-04T09:51:03.522Z</v>
       </c>
-      <c r="P19" t="str">
+      <c r="Q19" t="str">
         <v>2026-09-04T11:41:49.865Z</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>576fbffe-152c-4052-834c-1d230af3784a</v>
+      </c>
+      <c r="B20" t="str">
+        <v>แก้ไขข้อมูลนายจ้าง</v>
+      </c>
+      <c r="C20" t="str">
+        <v>เพิ่มส่งสาเหตุการแก้ไขข้อมูลนายจ้าง</v>
+      </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
+      <c r="E20" t="str">
+        <v>Back End</v>
+      </c>
+      <c r="F20" t="str">
+        <v>2026-09-07</v>
+      </c>
+      <c r="G20" t="str">
+        <v>2026-09-09</v>
+      </c>
+      <c r="H20" t="str">
+        <v>2026-09-09</v>
+      </c>
+      <c r="I20" t="str">
+        <v/>
+      </c>
+      <c r="J20" t="str">
+        <v>0</v>
+      </c>
+      <c r="K20" t="str">
+        <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
+      </c>
+      <c r="L20" t="str">
+        <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
+      </c>
+      <c r="M20" t="str">
+        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+      </c>
+      <c r="N20" t="str">
+        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
+      </c>
+      <c r="O20" t="str">
+        <v/>
+      </c>
+      <c r="P20" t="str">
+        <v>2026-09-08T04:37:27.473Z</v>
+      </c>
+      <c r="Q20" t="str">
+        <v>2026-09-08T07:00:51.150Z</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>c1b2bc1d-f4c5-42ea-bdc8-4fdc41bfd8ee</v>
+      </c>
+      <c r="B21" t="str">
+        <v>รายงาน ค.1(1)</v>
+      </c>
+      <c r="C21" t="str">
+        <v/>
+      </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
+      <c r="E21" t="str">
+        <v>Back End</v>
+      </c>
+      <c r="F21" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
+      <c r="H21" t="str">
+        <v>2026-09-09</v>
+      </c>
+      <c r="I21" t="str">
+        <v/>
+      </c>
+      <c r="J21" t="str">
+        <v>0</v>
+      </c>
+      <c r="K21" t="str">
+        <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
+      </c>
+      <c r="L21" t="str">
+        <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
+      </c>
+      <c r="M21" t="str">
+        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+      </c>
+      <c r="N21" t="str">
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+      </c>
+      <c r="O21" t="str">
+        <v/>
+      </c>
+      <c r="P21" t="str">
+        <v>2026-09-08T07:22:24.608Z</v>
+      </c>
+      <c r="Q21" t="str">
+        <v>2026-09-08T07:32:57.581Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q21"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I40"/>
+  <dimension ref="A1:I48"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3237,9 +3481,241 @@
         <v>2026-09-04T12:29:28.731Z</v>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>4a0e911b-d14b-4dcb-8e94-434265cc82ce</v>
+      </c>
+      <c r="B41" t="str">
+        <v>6ac09b86-b7ee-4b62-b048-4594eca71b6c</v>
+      </c>
+      <c r="C41" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="E41" t="str">
+        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+      </c>
+      <c r="F41" t="str">
+        <v>In Progress</v>
+      </c>
+      <c r="G41" t="str">
+        <v>2026-09-08T03:12:47.685Z</v>
+      </c>
+      <c r="H41" t="str">
+        <v>2026-09-08T03:12:47.689Z</v>
+      </c>
+      <c r="I41" t="str">
+        <v>2026-09-08T03:12:47.689Z</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>caa0b081-2da2-42d1-8a41-637b7852dc35</v>
+      </c>
+      <c r="B42" t="str">
+        <v>58f112bb-1a6e-4e26-8d8a-9bcd3e5bc31d</v>
+      </c>
+      <c r="C42" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="E42" t="str">
+        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+      </c>
+      <c r="F42" t="str">
+        <v>In Progress</v>
+      </c>
+      <c r="G42" t="str">
+        <v>2026-09-08T03:13:20.301Z</v>
+      </c>
+      <c r="H42" t="str">
+        <v>2026-09-08T03:13:20.304Z</v>
+      </c>
+      <c r="I42" t="str">
+        <v>2026-09-08T03:13:20.304Z</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>51130ead-6874-422e-872d-0d4dc7cedd2a</v>
+      </c>
+      <c r="B43" t="str">
+        <v>12f8c884-7a9e-4086-8352-ace2ea778248</v>
+      </c>
+      <c r="C43" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="E43" t="str">
+        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+      </c>
+      <c r="F43" t="str">
+        <v>In Progress</v>
+      </c>
+      <c r="G43" t="str">
+        <v>2026-09-08T03:13:32.551Z</v>
+      </c>
+      <c r="H43" t="str">
+        <v>2026-09-08T03:13:32.554Z</v>
+      </c>
+      <c r="I43" t="str">
+        <v>2026-09-08T03:13:32.554Z</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>af6be5e0-8805-4dfa-957f-2f280fd6664b</v>
+      </c>
+      <c r="B44" t="str">
+        <v>576fbffe-152c-4052-834c-1d230af3784a</v>
+      </c>
+      <c r="C44" t="str">
+        <v/>
+      </c>
+      <c r="D44" t="str">
+        <v/>
+      </c>
+      <c r="E44" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="F44" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="G44" t="str">
+        <v>2026-09-08T04:37:27.527Z</v>
+      </c>
+      <c r="H44" t="str">
+        <v>2026-09-08T04:37:27.530Z</v>
+      </c>
+      <c r="I44" t="str">
+        <v>2026-09-08T04:37:27.530Z</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>1c01001b-dc4a-4771-8bfd-39bac5b20ae2</v>
+      </c>
+      <c r="B45" t="str">
+        <v>a4db697d-4d50-4200-8355-647ab86cd480</v>
+      </c>
+      <c r="C45" t="str">
+        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+      </c>
+      <c r="D45" t="str">
+        <v>In Progress</v>
+      </c>
+      <c r="E45" t="str">
+        <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
+      </c>
+      <c r="F45" t="str">
+        <v>UAT</v>
+      </c>
+      <c r="G45" t="str">
+        <v>2026-09-08T07:00:11.958Z</v>
+      </c>
+      <c r="H45" t="str">
+        <v>2026-09-08T07:00:11.961Z</v>
+      </c>
+      <c r="I45" t="str">
+        <v>2026-09-08T07:00:11.961Z</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>03e95a8b-32af-4ff6-bfa9-ccf473e106ed</v>
+      </c>
+      <c r="B46" t="str">
+        <v>576fbffe-152c-4052-834c-1d230af3784a</v>
+      </c>
+      <c r="C46" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="E46" t="str">
+        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+      </c>
+      <c r="F46" t="str">
+        <v>In Progress</v>
+      </c>
+      <c r="G46" t="str">
+        <v>2026-09-08T07:00:40.996Z</v>
+      </c>
+      <c r="H46" t="str">
+        <v>2026-09-08T07:00:41.000Z</v>
+      </c>
+      <c r="I46" t="str">
+        <v>2026-09-08T07:00:41.000Z</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>21e3a036-dc27-42fa-a8b3-685611fc2c6b</v>
+      </c>
+      <c r="B47" t="str">
+        <v>c1b2bc1d-f4c5-42ea-bdc8-4fdc41bfd8ee</v>
+      </c>
+      <c r="C47" t="str">
+        <v/>
+      </c>
+      <c r="D47" t="str">
+        <v/>
+      </c>
+      <c r="E47" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="F47" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="G47" t="str">
+        <v>2026-09-08T07:22:24.666Z</v>
+      </c>
+      <c r="H47" t="str">
+        <v>2026-09-08T07:22:24.669Z</v>
+      </c>
+      <c r="I47" t="str">
+        <v>2026-09-08T07:22:24.669Z</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>a0f81578-a471-4805-b274-be597811c326</v>
+      </c>
+      <c r="B48" t="str">
+        <v>c1b2bc1d-f4c5-42ea-bdc8-4fdc41bfd8ee</v>
+      </c>
+      <c r="C48" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="E48" t="str">
+        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+      </c>
+      <c r="F48" t="str">
+        <v>In Progress</v>
+      </c>
+      <c r="G48" t="str">
+        <v>2026-09-08T07:22:32.102Z</v>
+      </c>
+      <c r="H48" t="str">
+        <v>2026-09-08T07:22:32.105Z</v>
+      </c>
+      <c r="I48" t="str">
+        <v>2026-09-08T07:22:32.105Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I40"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I48"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3487,7 +3963,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F34"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3511,10 +3987,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>ac8d7692-2e18-4474-b43d-1e1b085c3b72</v>
+        <v>0f184845-2a39-46bf-84af-9f5d02bff128</v>
       </c>
       <c r="B2" t="str">
-        <v>a4db697d-4d50-4200-8355-647ab86cd480</v>
+        <v>62533ab0-8ef1-45b9-b2d4-961570759b92</v>
       </c>
       <c r="C2" t="str">
         <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
@@ -3523,178 +3999,178 @@
         <v>0</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-09-04T09:40:35.742Z</v>
+        <v>2026-09-04T09:40:43.614Z</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-09-04T09:40:35.742Z</v>
+        <v>2026-09-04T09:40:43.614Z</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>0f184845-2a39-46bf-84af-9f5d02bff128</v>
+        <v>c13e3849-4301-4544-9fc0-32ab223dcf3a</v>
       </c>
       <c r="B3" t="str">
         <v>62533ab0-8ef1-45b9-b2d4-961570759b92</v>
       </c>
       <c r="C3" t="str">
-        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
+        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
       </c>
       <c r="D3" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3" t="str">
-        <v>2026-09-04T09:40:43.614Z</v>
+        <v>2026-09-04T09:40:43.621Z</v>
       </c>
       <c r="F3" t="str">
-        <v>2026-09-04T09:40:43.614Z</v>
+        <v>2026-09-04T09:40:43.621Z</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>c13e3849-4301-4544-9fc0-32ab223dcf3a</v>
+        <v>37e08404-2713-4dfe-936f-5f9322fa20e9</v>
       </c>
       <c r="B4" t="str">
-        <v>62533ab0-8ef1-45b9-b2d4-961570759b92</v>
+        <v>e0e2d398-49d2-4dc3-9fbc-512e2b97e4f5</v>
       </c>
       <c r="C4" t="str">
-        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
       <c r="D4" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4" t="str">
-        <v>2026-09-04T09:40:43.621Z</v>
+        <v>2026-09-04T09:41:08.413Z</v>
       </c>
       <c r="F4" t="str">
-        <v>2026-09-04T09:40:43.621Z</v>
+        <v>2026-09-04T09:41:08.413Z</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>37e08404-2713-4dfe-936f-5f9322fa20e9</v>
+        <v>c0934984-06c6-4ba5-9f45-c1b6e448bdbb</v>
       </c>
       <c r="B5" t="str">
         <v>e0e2d398-49d2-4dc3-9fbc-512e2b97e4f5</v>
       </c>
       <c r="C5" t="str">
-        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
       </c>
       <c r="D5" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" t="str">
-        <v>2026-09-04T09:41:08.413Z</v>
+        <v>2026-09-04T09:41:08.419Z</v>
       </c>
       <c r="F5" t="str">
-        <v>2026-09-04T09:41:08.413Z</v>
+        <v>2026-09-04T09:41:08.419Z</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>c0934984-06c6-4ba5-9f45-c1b6e448bdbb</v>
+        <v>b81e12b4-20a5-4fc4-a514-50370afcac96</v>
       </c>
       <c r="B6" t="str">
-        <v>e0e2d398-49d2-4dc3-9fbc-512e2b97e4f5</v>
+        <v>1e95dc95-6f63-4810-9d57-8520eb9b42c5</v>
       </c>
       <c r="C6" t="str">
-        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
       <c r="D6" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E6" t="str">
-        <v>2026-09-04T09:41:08.419Z</v>
+        <v>2026-09-04T09:41:39.531Z</v>
       </c>
       <c r="F6" t="str">
-        <v>2026-09-04T09:41:08.419Z</v>
+        <v>2026-09-04T09:41:39.531Z</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>b81e12b4-20a5-4fc4-a514-50370afcac96</v>
+        <v>76c55ffd-5c72-475c-9448-e969b036b7c0</v>
       </c>
       <c r="B7" t="str">
-        <v>1e95dc95-6f63-4810-9d57-8520eb9b42c5</v>
+        <v>e5a48211-b75f-4be3-aeee-dde8da731c1e</v>
       </c>
       <c r="C7" t="str">
-        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
       </c>
       <c r="D7" t="str">
         <v>0</v>
       </c>
       <c r="E7" t="str">
-        <v>2026-09-04T09:41:39.531Z</v>
+        <v>2026-09-04T09:47:39.835Z</v>
       </c>
       <c r="F7" t="str">
-        <v>2026-09-04T09:41:39.531Z</v>
+        <v>2026-09-04T09:47:39.835Z</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>f8edc8fa-0fc6-44c4-a15c-14cfe4475d9e</v>
+        <v>689f964d-b216-40de-881b-605919cf6b35</v>
       </c>
       <c r="B8" t="str">
-        <v>58f112bb-1a6e-4e26-8d8a-9bcd3e5bc31d</v>
+        <v>e5a48211-b75f-4be3-aeee-dde8da731c1e</v>
       </c>
       <c r="C8" t="str">
-        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
       <c r="D8" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" t="str">
-        <v>2026-09-04T09:44:49.319Z</v>
+        <v>2026-09-04T09:47:39.839Z</v>
       </c>
       <c r="F8" t="str">
-        <v>2026-09-04T09:44:49.319Z</v>
+        <v>2026-09-04T09:47:39.839Z</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>e1211e67-dde9-4873-a96f-6985e7753170</v>
+        <v>be30c4c5-9550-4b85-8401-c243a2cc9973</v>
       </c>
       <c r="B9" t="str">
-        <v>58f112bb-1a6e-4e26-8d8a-9bcd3e5bc31d</v>
+        <v>2ee76ad4-4c3e-40be-9b97-9100e95fa1a7</v>
       </c>
       <c r="C9" t="str">
-        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
+        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
       </c>
       <c r="D9" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E9" t="str">
-        <v>2026-09-04T09:44:49.325Z</v>
+        <v>2026-09-04T09:48:58.065Z</v>
       </c>
       <c r="F9" t="str">
-        <v>2026-09-04T09:44:49.325Z</v>
+        <v>2026-09-04T09:48:58.065Z</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>5a79cab4-c5b3-4c96-8b5a-bf72005b39f2</v>
+        <v>6402d1cb-71a9-4249-9e8d-765a6d771490</v>
       </c>
       <c r="B10" t="str">
-        <v>6ac09b86-b7ee-4b62-b048-4594eca71b6c</v>
+        <v>2ee76ad4-4c3e-40be-9b97-9100e95fa1a7</v>
       </c>
       <c r="C10" t="str">
         <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
       </c>
       <c r="D10" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E10" t="str">
-        <v>2026-09-04T09:45:22.504Z</v>
+        <v>2026-09-04T09:48:58.069Z</v>
       </c>
       <c r="F10" t="str">
-        <v>2026-09-04T09:45:22.504Z</v>
+        <v>2026-09-04T09:48:58.069Z</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>e16d77fc-e33d-4c73-be58-b8a0016c902a</v>
+        <v>837b7f6d-8aa7-4477-a101-2bc781f457eb</v>
       </c>
       <c r="B11" t="str">
-        <v>12f8c884-7a9e-4086-8352-ace2ea778248</v>
+        <v>e49e5c13-9c33-449b-9c2c-3b48f3119d16</v>
       </c>
       <c r="C11" t="str">
         <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
@@ -3703,298 +4179,298 @@
         <v>0</v>
       </c>
       <c r="E11" t="str">
-        <v>2026-09-04T09:45:31.784Z</v>
+        <v>2026-09-04T10:15:31.431Z</v>
       </c>
       <c r="F11" t="str">
-        <v>2026-09-04T09:45:31.784Z</v>
+        <v>2026-09-04T10:15:31.431Z</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>76c55ffd-5c72-475c-9448-e969b036b7c0</v>
+        <v>7bac2115-77f1-401f-ba0e-824e6d60f4fd</v>
       </c>
       <c r="B12" t="str">
-        <v>e5a48211-b75f-4be3-aeee-dde8da731c1e</v>
+        <v>e323d9c8-295f-472c-93f3-fefc39655d80</v>
       </c>
       <c r="C12" t="str">
-        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
+        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
       </c>
       <c r="D12" t="str">
         <v>0</v>
       </c>
       <c r="E12" t="str">
-        <v>2026-09-04T09:47:39.835Z</v>
+        <v>2026-09-04T10:15:52.847Z</v>
       </c>
       <c r="F12" t="str">
-        <v>2026-09-04T09:47:39.835Z</v>
+        <v>2026-09-04T10:15:52.847Z</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>689f964d-b216-40de-881b-605919cf6b35</v>
+        <v>4e27d0ea-d725-4fd6-8af3-af70d286f196</v>
       </c>
       <c r="B13" t="str">
-        <v>e5a48211-b75f-4be3-aeee-dde8da731c1e</v>
+        <v>81722c13-7a3f-4789-a1ac-a70c472369e0</v>
       </c>
       <c r="C13" t="str">
-        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
       </c>
       <c r="D13" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E13" t="str">
-        <v>2026-09-04T09:47:39.839Z</v>
+        <v>2026-09-04T11:41:49.851Z</v>
       </c>
       <c r="F13" t="str">
-        <v>2026-09-04T09:47:39.839Z</v>
+        <v>2026-09-04T11:41:49.851Z</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>be30c4c5-9550-4b85-8401-c243a2cc9973</v>
+        <v>9c21d982-7ad7-4a32-8875-f8af532fdf47</v>
       </c>
       <c r="B14" t="str">
-        <v>2ee76ad4-4c3e-40be-9b97-9100e95fa1a7</v>
+        <v>81722c13-7a3f-4789-a1ac-a70c472369e0</v>
       </c>
       <c r="C14" t="str">
-        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
       <c r="D14" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="str">
-        <v>2026-09-04T09:48:58.065Z</v>
+        <v>2026-09-04T11:41:49.858Z</v>
       </c>
       <c r="F14" t="str">
-        <v>2026-09-04T09:48:58.065Z</v>
+        <v>2026-09-04T11:41:49.858Z</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>6402d1cb-71a9-4249-9e8d-765a6d771490</v>
+        <v>61cb483a-a74d-4d8f-b675-5383b14f8f77</v>
       </c>
       <c r="B15" t="str">
-        <v>2ee76ad4-4c3e-40be-9b97-9100e95fa1a7</v>
+        <v>efd54252-a5fb-4a92-ae20-141a96834757</v>
       </c>
       <c r="C15" t="str">
-        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
+        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
       </c>
       <c r="D15" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15" t="str">
-        <v>2026-09-04T09:48:58.069Z</v>
+        <v>2026-09-04T12:29:03.469Z</v>
       </c>
       <c r="F15" t="str">
-        <v>2026-09-04T09:48:58.069Z</v>
+        <v>2026-09-04T12:29:03.469Z</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>837b7f6d-8aa7-4477-a101-2bc781f457eb</v>
+        <v>fe14404c-70ae-4023-afd5-86198706c46a</v>
       </c>
       <c r="B16" t="str">
-        <v>e49e5c13-9c33-449b-9c2c-3b48f3119d16</v>
+        <v>efd54252-a5fb-4a92-ae20-141a96834757</v>
       </c>
       <c r="C16" t="str">
-        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
       <c r="D16" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E16" t="str">
-        <v>2026-09-04T10:15:31.431Z</v>
+        <v>2026-09-04T12:29:03.477Z</v>
       </c>
       <c r="F16" t="str">
-        <v>2026-09-04T10:15:31.431Z</v>
+        <v>2026-09-04T12:29:03.477Z</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>7bac2115-77f1-401f-ba0e-824e6d60f4fd</v>
+        <v>5d381f35-c77e-4b8f-a9e7-4cbd4a8a52e8</v>
       </c>
       <c r="B17" t="str">
-        <v>e323d9c8-295f-472c-93f3-fefc39655d80</v>
+        <v>b5647f0e-4c20-454b-b334-30c5458df783</v>
       </c>
       <c r="C17" t="str">
-        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
+        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
       </c>
       <c r="D17" t="str">
         <v>0</v>
       </c>
       <c r="E17" t="str">
-        <v>2026-09-04T10:15:52.847Z</v>
+        <v>2026-09-04T12:29:08.635Z</v>
       </c>
       <c r="F17" t="str">
-        <v>2026-09-04T10:15:52.847Z</v>
+        <v>2026-09-04T12:29:08.635Z</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>4e27d0ea-d725-4fd6-8af3-af70d286f196</v>
+        <v>13efe219-b0c8-4dd9-82ca-e72d52723c88</v>
       </c>
       <c r="B18" t="str">
-        <v>81722c13-7a3f-4789-a1ac-a70c472369e0</v>
+        <v>b5647f0e-4c20-454b-b334-30c5458df783</v>
       </c>
       <c r="C18" t="str">
-        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
       <c r="D18" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E18" t="str">
-        <v>2026-09-04T11:41:49.851Z</v>
+        <v>2026-09-04T12:29:08.641Z</v>
       </c>
       <c r="F18" t="str">
-        <v>2026-09-04T11:41:49.851Z</v>
+        <v>2026-09-04T12:29:08.641Z</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>9c21d982-7ad7-4a32-8875-f8af532fdf47</v>
+        <v>cff700c0-46bf-44de-83d8-60c73d4565d6</v>
       </c>
       <c r="B19" t="str">
-        <v>81722c13-7a3f-4789-a1ac-a70c472369e0</v>
+        <v>2982e690-f17b-4b39-8695-ca1ad2d39f5e</v>
       </c>
       <c r="C19" t="str">
-        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+        <v>55d6e756-c40c-4755-84ab-c3458437acd6</v>
       </c>
       <c r="D19" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E19" t="str">
-        <v>2026-09-04T11:41:49.858Z</v>
+        <v>2026-09-04T12:29:13.365Z</v>
       </c>
       <c r="F19" t="str">
-        <v>2026-09-04T11:41:49.858Z</v>
+        <v>2026-09-04T12:29:13.365Z</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>61cb483a-a74d-4d8f-b675-5383b14f8f77</v>
+        <v>db8acf76-4830-485d-9ee7-4300a8abc346</v>
       </c>
       <c r="B20" t="str">
-        <v>efd54252-a5fb-4a92-ae20-141a96834757</v>
+        <v>2982e690-f17b-4b39-8695-ca1ad2d39f5e</v>
       </c>
       <c r="C20" t="str">
-        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
       <c r="D20" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" t="str">
-        <v>2026-09-04T12:29:03.469Z</v>
+        <v>2026-09-04T12:29:13.371Z</v>
       </c>
       <c r="F20" t="str">
-        <v>2026-09-04T12:29:03.469Z</v>
+        <v>2026-09-04T12:29:13.371Z</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>fe14404c-70ae-4023-afd5-86198706c46a</v>
+        <v>a0bde16c-883f-435d-a1e6-3ff8173e27fc</v>
       </c>
       <c r="B21" t="str">
-        <v>efd54252-a5fb-4a92-ae20-141a96834757</v>
+        <v>b1e061e4-cef5-46b4-a149-31d4340bd038</v>
       </c>
       <c r="C21" t="str">
-        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
       </c>
       <c r="D21" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E21" t="str">
-        <v>2026-09-04T12:29:03.477Z</v>
+        <v>2026-09-04T12:29:18.501Z</v>
       </c>
       <c r="F21" t="str">
-        <v>2026-09-04T12:29:03.477Z</v>
+        <v>2026-09-04T12:29:18.501Z</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>5d381f35-c77e-4b8f-a9e7-4cbd4a8a52e8</v>
+        <v>35763cf5-1687-4782-a94f-47223bc94f62</v>
       </c>
       <c r="B22" t="str">
-        <v>b5647f0e-4c20-454b-b334-30c5458df783</v>
+        <v>b1e061e4-cef5-46b4-a149-31d4340bd038</v>
       </c>
       <c r="C22" t="str">
-        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
+        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
       </c>
       <c r="D22" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E22" t="str">
-        <v>2026-09-04T12:29:08.635Z</v>
+        <v>2026-09-04T12:29:18.507Z</v>
       </c>
       <c r="F22" t="str">
-        <v>2026-09-04T12:29:08.635Z</v>
+        <v>2026-09-04T12:29:18.507Z</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>13efe219-b0c8-4dd9-82ca-e72d52723c88</v>
+        <v>035c1398-3263-4e99-8273-9aba0c9023ba</v>
       </c>
       <c r="B23" t="str">
-        <v>b5647f0e-4c20-454b-b334-30c5458df783</v>
+        <v>764fd6d8-3712-4019-8c67-6e3615085faf</v>
       </c>
       <c r="C23" t="str">
-        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
       </c>
       <c r="D23" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E23" t="str">
-        <v>2026-09-04T12:29:08.641Z</v>
+        <v>2026-09-04T12:29:22.908Z</v>
       </c>
       <c r="F23" t="str">
-        <v>2026-09-04T12:29:08.641Z</v>
+        <v>2026-09-04T12:29:22.908Z</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>cff700c0-46bf-44de-83d8-60c73d4565d6</v>
+        <v>544f63ce-d992-4c80-aaac-33a8fa860614</v>
       </c>
       <c r="B24" t="str">
-        <v>2982e690-f17b-4b39-8695-ca1ad2d39f5e</v>
+        <v>764fd6d8-3712-4019-8c67-6e3615085faf</v>
       </c>
       <c r="C24" t="str">
-        <v>55d6e756-c40c-4755-84ab-c3458437acd6</v>
+        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
       </c>
       <c r="D24" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E24" t="str">
-        <v>2026-09-04T12:29:13.365Z</v>
+        <v>2026-09-04T12:29:22.912Z</v>
       </c>
       <c r="F24" t="str">
-        <v>2026-09-04T12:29:13.365Z</v>
+        <v>2026-09-04T12:29:22.912Z</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>db8acf76-4830-485d-9ee7-4300a8abc346</v>
+        <v>5da43984-fa10-419d-be97-55c04f991d54</v>
       </c>
       <c r="B25" t="str">
-        <v>2982e690-f17b-4b39-8695-ca1ad2d39f5e</v>
+        <v>d6acd7ea-e69f-4894-9ce4-c8ae86da6bd2</v>
       </c>
       <c r="C25" t="str">
-        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+        <v>55d6e756-c40c-4755-84ab-c3458437acd6</v>
       </c>
       <c r="D25" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E25" t="str">
-        <v>2026-09-04T12:29:13.371Z</v>
+        <v>2026-09-04T12:29:28.748Z</v>
       </c>
       <c r="F25" t="str">
-        <v>2026-09-04T12:29:13.371Z</v>
+        <v>2026-09-04T12:29:28.748Z</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>a0bde16c-883f-435d-a1e6-3ff8173e27fc</v>
+        <v>9c43d17e-fee0-4a90-b4b0-7076e3a5fda9</v>
       </c>
       <c r="B26" t="str">
-        <v>b1e061e4-cef5-46b4-a149-31d4340bd038</v>
+        <v>a4db697d-4d50-4200-8355-647ab86cd480</v>
       </c>
       <c r="C26" t="str">
         <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
@@ -4003,95 +4479,175 @@
         <v>0</v>
       </c>
       <c r="E26" t="str">
-        <v>2026-09-04T12:29:18.501Z</v>
+        <v>2026-09-08T02:27:47.879Z</v>
       </c>
       <c r="F26" t="str">
-        <v>2026-09-04T12:29:18.501Z</v>
+        <v>2026-09-08T02:27:47.879Z</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>35763cf5-1687-4782-a94f-47223bc94f62</v>
+        <v>2c1e3965-52ed-4324-98bc-d48def9e2254</v>
       </c>
       <c r="B27" t="str">
-        <v>b1e061e4-cef5-46b4-a149-31d4340bd038</v>
+        <v>a4db697d-4d50-4200-8355-647ab86cd480</v>
       </c>
       <c r="C27" t="str">
-        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
       <c r="D27" t="str">
         <v>1</v>
       </c>
       <c r="E27" t="str">
-        <v>2026-09-04T12:29:18.507Z</v>
+        <v>2026-09-08T02:27:47.888Z</v>
       </c>
       <c r="F27" t="str">
-        <v>2026-09-04T12:29:18.507Z</v>
+        <v>2026-09-08T02:27:47.888Z</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>035c1398-3263-4e99-8273-9aba0c9023ba</v>
+        <v>2030cc27-64e7-4348-a193-88c452d06ec4</v>
       </c>
       <c r="B28" t="str">
-        <v>764fd6d8-3712-4019-8c67-6e3615085faf</v>
+        <v>6ac09b86-b7ee-4b62-b048-4594eca71b6c</v>
       </c>
       <c r="C28" t="str">
-        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
+        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
       </c>
       <c r="D28" t="str">
         <v>0</v>
       </c>
       <c r="E28" t="str">
-        <v>2026-09-04T12:29:22.908Z</v>
+        <v>2026-09-08T03:12:47.728Z</v>
       </c>
       <c r="F28" t="str">
-        <v>2026-09-04T12:29:22.908Z</v>
+        <v>2026-09-08T03:12:47.728Z</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>544f63ce-d992-4c80-aaac-33a8fa860614</v>
+        <v>b3b7233e-4aaf-4596-aa01-e044607b2861</v>
       </c>
       <c r="B29" t="str">
-        <v>764fd6d8-3712-4019-8c67-6e3615085faf</v>
+        <v>12f8c884-7a9e-4086-8352-ace2ea778248</v>
       </c>
       <c r="C29" t="str">
-        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
+        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
       </c>
       <c r="D29" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E29" t="str">
-        <v>2026-09-04T12:29:22.912Z</v>
+        <v>2026-09-08T03:13:32.577Z</v>
       </c>
       <c r="F29" t="str">
-        <v>2026-09-04T12:29:22.912Z</v>
+        <v>2026-09-08T03:13:32.577Z</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>5da43984-fa10-419d-be97-55c04f991d54</v>
+        <v>ba8ae40b-58f0-4048-a945-af20bbc3f415</v>
       </c>
       <c r="B30" t="str">
-        <v>d6acd7ea-e69f-4894-9ce4-c8ae86da6bd2</v>
+        <v>58f112bb-1a6e-4e26-8d8a-9bcd3e5bc31d</v>
       </c>
       <c r="C30" t="str">
-        <v>55d6e756-c40c-4755-84ab-c3458437acd6</v>
+        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
       </c>
       <c r="D30" t="str">
         <v>0</v>
       </c>
       <c r="E30" t="str">
-        <v>2026-09-04T12:29:28.748Z</v>
+        <v>2026-09-08T07:00:38.362Z</v>
       </c>
       <c r="F30" t="str">
-        <v>2026-09-04T12:29:28.748Z</v>
+        <v>2026-09-08T07:00:38.362Z</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>49b20734-492a-4950-9f99-ef820a888dc0</v>
+      </c>
+      <c r="B31" t="str">
+        <v>58f112bb-1a6e-4e26-8d8a-9bcd3e5bc31d</v>
+      </c>
+      <c r="C31" t="str">
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+      </c>
+      <c r="D31" t="str">
+        <v>1</v>
+      </c>
+      <c r="E31" t="str">
+        <v>2026-09-08T07:00:38.372Z</v>
+      </c>
+      <c r="F31" t="str">
+        <v>2026-09-08T07:00:38.372Z</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>dee4af21-e9a1-40ae-b72a-dcbf02909835</v>
+      </c>
+      <c r="B32" t="str">
+        <v>576fbffe-152c-4052-834c-1d230af3784a</v>
+      </c>
+      <c r="C32" t="str">
+        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
+      </c>
+      <c r="D32" t="str">
+        <v>0</v>
+      </c>
+      <c r="E32" t="str">
+        <v>2026-09-08T07:00:51.130Z</v>
+      </c>
+      <c r="F32" t="str">
+        <v>2026-09-08T07:00:51.130Z</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>9caf7a0a-46c6-4476-b1df-0b18e5e53d52</v>
+      </c>
+      <c r="B33" t="str">
+        <v>576fbffe-152c-4052-834c-1d230af3784a</v>
+      </c>
+      <c r="C33" t="str">
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+      </c>
+      <c r="D33" t="str">
+        <v>1</v>
+      </c>
+      <c r="E33" t="str">
+        <v>2026-09-08T07:00:51.140Z</v>
+      </c>
+      <c r="F33" t="str">
+        <v>2026-09-08T07:00:51.140Z</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>ca84d7b2-4097-412c-a221-df5574d728c3</v>
+      </c>
+      <c r="B34" t="str">
+        <v>c1b2bc1d-f4c5-42ea-bdc8-4fdc41bfd8ee</v>
+      </c>
+      <c r="C34" t="str">
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+      </c>
+      <c r="D34" t="str">
+        <v>0</v>
+      </c>
+      <c r="E34" t="str">
+        <v>2026-09-08T07:22:32.129Z</v>
+      </c>
+      <c r="F34" t="str">
+        <v>2026-09-08T07:22:32.129Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F30"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F34"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: enhance task card UI with overdue state indication
- Integrated overdue detection into the TaskCard component, utilizing the new `getTaskOverdueState` function.
- Updated visual styles to highlight overdue tasks with distinct colors and labels.
- Refactored date display logic to accommodate overdue conditions, improving user experience.
- Adjusted utility functions to ensure accurate overdue checks across task management features.
- Updated taskDB.xlsx to reflect changes in task attributes and overdue handling.
</commit_message>
<xml_diff>
--- a/data/taskDB.xlsx
+++ b/data/taskDB.xlsx
@@ -804,7 +804,7 @@
         <v>2026-09-01T07:23:24.979Z</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-09-08T07:44:34.904Z</v>
+        <v>2026-09-09T03:54:06.026Z</v>
       </c>
     </row>
     <row r="3">
@@ -824,7 +824,7 @@
         <v>2026-09-01T07:23:24.981Z</v>
       </c>
       <c r="F3" t="str">
-        <v>2026-09-08T07:44:34.911Z</v>
+        <v>2026-09-09T03:54:06.029Z</v>
       </c>
     </row>
     <row r="4">
@@ -844,7 +844,7 @@
         <v>2026-09-01T07:23:24.983Z</v>
       </c>
       <c r="F4" t="str">
-        <v>2026-09-08T07:44:34.925Z</v>
+        <v>2026-09-09T03:54:06.037Z</v>
       </c>
     </row>
     <row r="5">
@@ -864,7 +864,7 @@
         <v>2026-09-01T07:23:24.985Z</v>
       </c>
       <c r="F5" t="str">
-        <v>2026-09-08T07:44:34.917Z</v>
+        <v>2026-09-09T03:54:06.033Z</v>
       </c>
     </row>
     <row r="6">
@@ -884,7 +884,7 @@
         <v>2026-09-01T07:23:24.988Z</v>
       </c>
       <c r="F6" t="str">
-        <v>2026-09-08T07:44:34.932Z</v>
+        <v>2026-09-09T03:54:06.041Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: enhance status management with editing capabilities
- Added functionality to edit existing statuses, including validation for reserved names.
- Updated the SettingsDialog component to support editing status names and colors.
- Implemented error handling for attempts to modify default statuses.
- Enhanced UI to reflect editing state and provide user feedback during status updates.
- Updated taskDB.xlsx to include changes related to status management.
</commit_message>
<xml_diff>
--- a/data/taskDB.xlsx
+++ b/data/taskDB.xlsx
@@ -463,7 +463,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -665,9 +665,49 @@
         <v>2026-09-04T11:41:47.465Z</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>18a4faac-4efd-4b46-ac5b-1888d942a675</v>
+      </c>
+      <c r="B11" t="str">
+        <v>30680aff-dffc-4170-9152-67ee539b3e93</v>
+      </c>
+      <c r="C11" t="str">
+        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
+      </c>
+      <c r="D11" t="str">
+        <v>0</v>
+      </c>
+      <c r="E11" t="str">
+        <v>2026-09-11T06:55:12.829Z</v>
+      </c>
+      <c r="F11" t="str">
+        <v>2026-09-11T06:55:12.829Z</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>ee8bf0b0-933f-475c-a471-0ddfb283a833</v>
+      </c>
+      <c r="B12" t="str">
+        <v>ba295d36-7862-4119-9b75-ab172c89a88e</v>
+      </c>
+      <c r="C12" t="str">
+        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
+      </c>
+      <c r="D12" t="str">
+        <v>0</v>
+      </c>
+      <c r="E12" t="str">
+        <v>2026-09-11T06:56:01.912Z</v>
+      </c>
+      <c r="F12" t="str">
+        <v>2026-09-11T06:56:01.912Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F12"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -765,7 +805,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -804,7 +844,7 @@
         <v>2026-09-01T07:23:24.979Z</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-09-09T03:54:06.026Z</v>
+        <v>2026-09-11T07:10:49.660Z</v>
       </c>
     </row>
     <row r="3">
@@ -824,7 +864,7 @@
         <v>2026-09-01T07:23:24.981Z</v>
       </c>
       <c r="F3" t="str">
-        <v>2026-09-09T03:54:06.029Z</v>
+        <v>2026-09-11T07:10:49.664Z</v>
       </c>
     </row>
     <row r="4">
@@ -844,7 +884,7 @@
         <v>2026-09-01T07:23:24.983Z</v>
       </c>
       <c r="F4" t="str">
-        <v>2026-09-09T03:54:06.037Z</v>
+        <v>2026-09-11T07:10:49.671Z</v>
       </c>
     </row>
     <row r="5">
@@ -864,7 +904,7 @@
         <v>2026-09-01T07:23:24.985Z</v>
       </c>
       <c r="F5" t="str">
-        <v>2026-09-09T03:54:06.033Z</v>
+        <v>2026-09-11T07:10:49.667Z</v>
       </c>
     </row>
     <row r="6">
@@ -884,12 +924,32 @@
         <v>2026-09-01T07:23:24.988Z</v>
       </c>
       <c r="F6" t="str">
-        <v>2026-09-09T03:54:06.041Z</v>
+        <v>2026-09-11T07:10:49.675Z</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>f568698e-99c5-418d-8036-5f99072d6e28</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Fixing</v>
+      </c>
+      <c r="C7" t="str">
+        <v>#F7D83B</v>
+      </c>
+      <c r="D7" t="str">
+        <v>2</v>
+      </c>
+      <c r="E7" t="str">
+        <v>2026-09-11T06:54:30.253Z</v>
+      </c>
+      <c r="F7" t="str">
+        <v>2026-09-11T06:54:36.730Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1195,7 +1255,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q21"/>
+  <dimension ref="A1:Q25"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1538,10 +1598,10 @@
         <v>2026-09-04</v>
       </c>
       <c r="H7" t="str">
-        <v>2026-09-02</v>
+        <v>2026-09-14</v>
       </c>
       <c r="I7" t="str">
-        <v/>
+        <v>2026-09-16</v>
       </c>
       <c r="J7" t="str">
         <v>0</v>
@@ -1553,7 +1613,7 @@
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
       <c r="M7" t="str">
-        <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
+        <v>f568698e-99c5-418d-8036-5f99072d6e28</v>
       </c>
       <c r="N7" t="str">
         <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
@@ -1565,7 +1625,7 @@
         <v>2026-09-04T09:27:00.612Z</v>
       </c>
       <c r="Q7" t="str">
-        <v>2026-09-04T11:32:30.909Z</v>
+        <v>2026-09-11T06:56:21.637Z</v>
       </c>
     </row>
     <row r="8">
@@ -1594,7 +1654,7 @@
         <v>2026-09-02</v>
       </c>
       <c r="I8" t="str">
-        <v/>
+        <v>2026-09-13</v>
       </c>
       <c r="J8" t="str">
         <v>0</v>
@@ -1618,7 +1678,7 @@
         <v>2026-09-04T09:29:47.993Z</v>
       </c>
       <c r="Q8" t="str">
-        <v>2026-09-04T09:41:39.538Z</v>
+        <v>2026-09-11T06:49:45.510Z</v>
       </c>
     </row>
     <row r="9">
@@ -1871,7 +1931,7 @@
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
       <c r="M13" t="str">
-        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+        <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
       </c>
       <c r="N13" t="str">
         <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
@@ -1883,7 +1943,7 @@
         <v>2026-09-04T09:43:36.886Z</v>
       </c>
       <c r="Q13" t="str">
-        <v>2026-09-08T03:13:32.587Z</v>
+        <v>2026-09-09T10:31:25.123Z</v>
       </c>
     </row>
     <row r="14">
@@ -1912,7 +1972,7 @@
         <v>2026-09-09</v>
       </c>
       <c r="I14" t="str">
-        <v/>
+        <v>2026-09-20</v>
       </c>
       <c r="J14" t="str">
         <v>0</v>
@@ -1924,7 +1984,7 @@
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
       <c r="M14" t="str">
-        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+        <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
       </c>
       <c r="N14" t="str">
         <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
@@ -1936,7 +1996,7 @@
         <v>2026-09-04T09:43:56.520Z</v>
       </c>
       <c r="Q14" t="str">
-        <v>2026-09-08T03:12:47.743Z</v>
+        <v>2026-09-11T06:58:59.742Z</v>
       </c>
     </row>
     <row r="15">
@@ -1977,7 +2037,7 @@
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
       <c r="M15" t="str">
-        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+        <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
       </c>
       <c r="N15" t="str">
         <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
@@ -1989,7 +2049,7 @@
         <v>2026-09-04T09:44:42.509Z</v>
       </c>
       <c r="Q15" t="str">
-        <v>2026-09-08T07:00:38.382Z</v>
+        <v>2026-09-11T06:48:29.153Z</v>
       </c>
     </row>
     <row r="16">
@@ -2230,7 +2290,7 @@
         <v>2026-09-09</v>
       </c>
       <c r="I20" t="str">
-        <v/>
+        <v>2026-09-13</v>
       </c>
       <c r="J20" t="str">
         <v>0</v>
@@ -2242,7 +2302,7 @@
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
       <c r="M20" t="str">
-        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+        <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
       </c>
       <c r="N20" t="str">
         <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
@@ -2254,7 +2314,7 @@
         <v>2026-09-08T04:37:27.473Z</v>
       </c>
       <c r="Q20" t="str">
-        <v>2026-09-08T07:00:51.150Z</v>
+        <v>2026-09-11T06:48:10.776Z</v>
       </c>
     </row>
     <row r="21">
@@ -2283,7 +2343,7 @@
         <v>2026-09-09</v>
       </c>
       <c r="I21" t="str">
-        <v/>
+        <v>2026-09-13</v>
       </c>
       <c r="J21" t="str">
         <v>0</v>
@@ -2295,7 +2355,7 @@
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
       <c r="M21" t="str">
-        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+        <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
       </c>
       <c r="N21" t="str">
         <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
@@ -2307,19 +2367,233 @@
         <v>2026-09-08T07:22:24.608Z</v>
       </c>
       <c r="Q21" t="str">
-        <v>2026-09-08T07:32:57.581Z</v>
+        <v>2026-09-11T06:48:04.045Z</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>a2d08247-d1c8-4c29-9663-96adb51418ff</v>
+      </c>
+      <c r="B22" t="str">
+        <v xml:space="preserve">Statement </v>
+      </c>
+      <c r="C22" t="str">
+        <v>กดรับกรณี 1 รายการ มีหลายเลขอ้างอิง</v>
+      </c>
+      <c r="D22" t="str">
+        <v/>
+      </c>
+      <c r="E22" t="str">
+        <v>Back End</v>
+      </c>
+      <c r="F22" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="G22" t="str">
+        <v/>
+      </c>
+      <c r="H22" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="I22" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="J22" t="str">
+        <v>0</v>
+      </c>
+      <c r="K22" t="str">
+        <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
+      </c>
+      <c r="L22" t="str">
+        <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
+      </c>
+      <c r="M22" t="str">
+        <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
+      </c>
+      <c r="N22" t="str">
+        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
+      </c>
+      <c r="O22" t="str">
+        <v/>
+      </c>
+      <c r="P22" t="str">
+        <v>2026-09-11T06:49:21.261Z</v>
+      </c>
+      <c r="Q22" t="str">
+        <v>2026-09-11T06:49:25.747Z</v>
+      </c>
+    </row>
+    <row r="23" xml:space="preserve">
+      <c r="A23" t="str">
+        <v>61dd30f5-4dcd-42a8-a3f7-19c95b56a2fc</v>
+      </c>
+      <c r="B23" t="str">
+        <v>กรมธรรม์ทั้งหมด</v>
+      </c>
+      <c r="C23" t="str">
+        <v>เพิ่ม Filter ชื่อกรมธรรม์ (ใช้ชื่อตามรายงานส่งเงิน)</v>
+      </c>
+      <c r="D23" t="str" xml:space="preserve">
+        <v xml:space="preserve">BE เพิ่มเส้น get ค้นหาชื่อกรมธรรม์
+FE ต่อ api ยิงค้นหาชื่อกรมธรรม์ ปรับช่องราคาบัตรเป็น auto complete</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Back End</v>
+      </c>
+      <c r="F23" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="G23" t="str">
+        <v/>
+      </c>
+      <c r="H23" t="str">
+        <v>2026-09-14</v>
+      </c>
+      <c r="I23" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="J23" t="str">
+        <v>0</v>
+      </c>
+      <c r="K23" t="str">
+        <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
+      </c>
+      <c r="L23" t="str">
+        <v>3663067e-457b-445c-9656-3c5886a7d364</v>
+      </c>
+      <c r="M23" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="N23" t="str">
+        <v/>
+      </c>
+      <c r="O23" t="str">
+        <v/>
+      </c>
+      <c r="P23" t="str">
+        <v>2026-09-11T06:58:20.486Z</v>
+      </c>
+      <c r="Q23" t="str">
+        <v>2026-09-11T06:58:20.507Z</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>f503ee00-c9c6-4e8f-b72e-bc09d0fec90e</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Dashboard นำร่อง</v>
+      </c>
+      <c r="C24" t="str">
+        <v>เพิ่มการแสดงผลใบรับรองแพทย์พื้นที่นำร่องให้มี 3 สถานะใบรับรองแพทย์</v>
+      </c>
+      <c r="D24" t="str">
+        <v/>
+      </c>
+      <c r="E24" t="str">
+        <v>Back End</v>
+      </c>
+      <c r="F24" t="str">
+        <v/>
+      </c>
+      <c r="G24" t="str">
+        <v/>
+      </c>
+      <c r="H24" t="str">
+        <v>2026-08-22</v>
+      </c>
+      <c r="I24" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="J24" t="str">
+        <v>0</v>
+      </c>
+      <c r="K24" t="str">
+        <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
+      </c>
+      <c r="L24" t="str">
+        <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
+      </c>
+      <c r="M24" t="str">
+        <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
+      </c>
+      <c r="N24" t="str">
+        <v/>
+      </c>
+      <c r="O24" t="str">
+        <v/>
+      </c>
+      <c r="P24" t="str">
+        <v>2026-09-11T06:59:51.867Z</v>
+      </c>
+      <c r="Q24" t="str">
+        <v>2026-09-11T06:59:51.886Z</v>
+      </c>
+    </row>
+    <row r="25" xml:space="preserve">
+      <c r="A25" t="str">
+        <v>db57a402-f79a-4e85-9c0f-e0aa07395e56</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Dashboard นำร่อง</v>
+      </c>
+      <c r="C25" t="str" xml:space="preserve">
+        <v xml:space="preserve">เพิ่มการแสดงผลใบรับรองแพทย์พื้นที่นำร่องให้มีเพิ่มเติมรายละเอียดสถิติโรคผิดปกติ
+</v>
+      </c>
+      <c r="D25" t="str">
+        <v/>
+      </c>
+      <c r="E25" t="str">
+        <v>Back End</v>
+      </c>
+      <c r="F25" t="str">
+        <v>2026-09-01</v>
+      </c>
+      <c r="G25" t="str">
+        <v/>
+      </c>
+      <c r="H25" t="str">
+        <v>2026-09-14</v>
+      </c>
+      <c r="I25" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="J25" t="str">
+        <v>0</v>
+      </c>
+      <c r="K25" t="str">
+        <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
+      </c>
+      <c r="L25" t="str">
+        <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
+      </c>
+      <c r="M25" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="N25" t="str">
+        <v/>
+      </c>
+      <c r="O25" t="str">
+        <v/>
+      </c>
+      <c r="P25" t="str">
+        <v>2026-09-11T07:00:25.947Z</v>
+      </c>
+      <c r="Q25" t="str">
+        <v>2026-09-11T07:00:25.966Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q25"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I48"/>
+  <dimension ref="A1:I59"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3713,16 +3987,335 @@
         <v>2026-09-08T07:22:32.105Z</v>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>285d9520-4d21-46ee-bdbe-905894f8206c</v>
+      </c>
+      <c r="B49" t="str">
+        <v>576fbffe-152c-4052-834c-1d230af3784a</v>
+      </c>
+      <c r="C49" t="str">
+        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+      </c>
+      <c r="D49" t="str">
+        <v>In Progress</v>
+      </c>
+      <c r="E49" t="str">
+        <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
+      </c>
+      <c r="F49" t="str">
+        <v>UAT</v>
+      </c>
+      <c r="G49" t="str">
+        <v>2026-09-09T10:31:18.373Z</v>
+      </c>
+      <c r="H49" t="str">
+        <v>2026-09-09T10:31:18.386Z</v>
+      </c>
+      <c r="I49" t="str">
+        <v>2026-09-09T10:31:18.386Z</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>d619cea0-8bf9-4287-a1b4-6d6108d18ea5</v>
+      </c>
+      <c r="B50" t="str">
+        <v>c1b2bc1d-f4c5-42ea-bdc8-4fdc41bfd8ee</v>
+      </c>
+      <c r="C50" t="str">
+        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+      </c>
+      <c r="D50" t="str">
+        <v>In Progress</v>
+      </c>
+      <c r="E50" t="str">
+        <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
+      </c>
+      <c r="F50" t="str">
+        <v>UAT</v>
+      </c>
+      <c r="G50" t="str">
+        <v>2026-09-09T10:31:18.386Z</v>
+      </c>
+      <c r="H50" t="str">
+        <v>2026-09-09T10:31:18.400Z</v>
+      </c>
+      <c r="I50" t="str">
+        <v>2026-09-09T10:31:18.400Z</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>00c8160d-ee81-440d-a1b9-7a6ed5f7b08a</v>
+      </c>
+      <c r="B51" t="str">
+        <v>6ac09b86-b7ee-4b62-b048-4594eca71b6c</v>
+      </c>
+      <c r="C51" t="str">
+        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+      </c>
+      <c r="D51" t="str">
+        <v>In Progress</v>
+      </c>
+      <c r="E51" t="str">
+        <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
+      </c>
+      <c r="F51" t="str">
+        <v>UAT</v>
+      </c>
+      <c r="G51" t="str">
+        <v>2026-09-09T10:31:24.160Z</v>
+      </c>
+      <c r="H51" t="str">
+        <v>2026-09-09T10:31:24.164Z</v>
+      </c>
+      <c r="I51" t="str">
+        <v>2026-09-09T10:31:24.164Z</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>d84de3d8-8660-420f-a259-bbbcbe77eff0</v>
+      </c>
+      <c r="B52" t="str">
+        <v>12f8c884-7a9e-4086-8352-ace2ea778248</v>
+      </c>
+      <c r="C52" t="str">
+        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+      </c>
+      <c r="D52" t="str">
+        <v>In Progress</v>
+      </c>
+      <c r="E52" t="str">
+        <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
+      </c>
+      <c r="F52" t="str">
+        <v>UAT</v>
+      </c>
+      <c r="G52" t="str">
+        <v>2026-09-09T10:31:25.104Z</v>
+      </c>
+      <c r="H52" t="str">
+        <v>2026-09-09T10:31:25.109Z</v>
+      </c>
+      <c r="I52" t="str">
+        <v>2026-09-09T10:31:25.109Z</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>ac471f39-597a-4305-b9b1-451ce6a2cbe6</v>
+      </c>
+      <c r="B53" t="str">
+        <v>58f112bb-1a6e-4e26-8d8a-9bcd3e5bc31d</v>
+      </c>
+      <c r="C53" t="str">
+        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+      </c>
+      <c r="D53" t="str">
+        <v>In Progress</v>
+      </c>
+      <c r="E53" t="str">
+        <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
+      </c>
+      <c r="F53" t="str">
+        <v>UAT</v>
+      </c>
+      <c r="G53" t="str">
+        <v>2026-09-11T06:48:29.134Z</v>
+      </c>
+      <c r="H53" t="str">
+        <v>2026-09-11T06:48:29.139Z</v>
+      </c>
+      <c r="I53" t="str">
+        <v>2026-09-11T06:48:29.139Z</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>da0d49ed-678e-4ae1-9e2b-1ffbda3fd584</v>
+      </c>
+      <c r="B54" t="str">
+        <v>a2d08247-d1c8-4c29-9663-96adb51418ff</v>
+      </c>
+      <c r="C54" t="str">
+        <v/>
+      </c>
+      <c r="D54" t="str">
+        <v/>
+      </c>
+      <c r="E54" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="F54" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="G54" t="str">
+        <v>2026-09-11T06:49:21.346Z</v>
+      </c>
+      <c r="H54" t="str">
+        <v>2026-09-11T06:49:21.352Z</v>
+      </c>
+      <c r="I54" t="str">
+        <v>2026-09-11T06:49:21.352Z</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>878784ae-75fc-41b8-8c0e-dffbc39f9786</v>
+      </c>
+      <c r="B55" t="str">
+        <v>a2d08247-d1c8-4c29-9663-96adb51418ff</v>
+      </c>
+      <c r="C55" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="D55" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="E55" t="str">
+        <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
+      </c>
+      <c r="F55" t="str">
+        <v>UAT</v>
+      </c>
+      <c r="G55" t="str">
+        <v>2026-09-11T06:49:25.730Z</v>
+      </c>
+      <c r="H55" t="str">
+        <v>2026-09-11T06:49:25.734Z</v>
+      </c>
+      <c r="I55" t="str">
+        <v>2026-09-11T06:49:25.734Z</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>c8df673c-eed1-4151-aa16-a0d61b6ebddd</v>
+      </c>
+      <c r="B56" t="str">
+        <v>e323d9c8-295f-472c-93f3-fefc39655d80</v>
+      </c>
+      <c r="C56" t="str">
+        <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
+      </c>
+      <c r="D56" t="str">
+        <v>UAT</v>
+      </c>
+      <c r="E56" t="str">
+        <v>f568698e-99c5-418d-8036-5f99072d6e28</v>
+      </c>
+      <c r="F56" t="str">
+        <v>Fixing</v>
+      </c>
+      <c r="G56" t="str">
+        <v>2026-09-11T06:54:44.163Z</v>
+      </c>
+      <c r="H56" t="str">
+        <v>2026-09-11T06:54:44.166Z</v>
+      </c>
+      <c r="I56" t="str">
+        <v>2026-09-11T06:54:44.166Z</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>0f4891be-1e6b-43ba-aa17-b79ac3758c9e</v>
+      </c>
+      <c r="B57" t="str">
+        <v>61dd30f5-4dcd-42a8-a3f7-19c95b56a2fc</v>
+      </c>
+      <c r="C57" t="str">
+        <v/>
+      </c>
+      <c r="D57" t="str">
+        <v/>
+      </c>
+      <c r="E57" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="F57" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="G57" t="str">
+        <v>2026-09-11T06:58:20.532Z</v>
+      </c>
+      <c r="H57" t="str">
+        <v>2026-09-11T06:58:20.536Z</v>
+      </c>
+      <c r="I57" t="str">
+        <v>2026-09-11T06:58:20.536Z</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>4fe23135-e4ba-4ba8-8a2d-4e6e7e7b6a10</v>
+      </c>
+      <c r="B58" t="str">
+        <v>f503ee00-c9c6-4e8f-b72e-bc09d0fec90e</v>
+      </c>
+      <c r="C58" t="str">
+        <v/>
+      </c>
+      <c r="D58" t="str">
+        <v/>
+      </c>
+      <c r="E58" t="str">
+        <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
+      </c>
+      <c r="F58" t="str">
+        <v>UAT</v>
+      </c>
+      <c r="G58" t="str">
+        <v>2026-09-11T06:59:51.914Z</v>
+      </c>
+      <c r="H58" t="str">
+        <v>2026-09-11T06:59:51.918Z</v>
+      </c>
+      <c r="I58" t="str">
+        <v>2026-09-11T06:59:51.918Z</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>33bb9a26-783b-467d-8b8f-99632611b187</v>
+      </c>
+      <c r="B59" t="str">
+        <v>db57a402-f79a-4e85-9c0f-e0aa07395e56</v>
+      </c>
+      <c r="C59" t="str">
+        <v/>
+      </c>
+      <c r="D59" t="str">
+        <v/>
+      </c>
+      <c r="E59" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="F59" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="G59" t="str">
+        <v>2026-09-11T07:00:25.991Z</v>
+      </c>
+      <c r="H59" t="str">
+        <v>2026-09-11T07:00:25.995Z</v>
+      </c>
+      <c r="I59" t="str">
+        <v>2026-09-11T07:00:25.995Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I48"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I59"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3954,16 +4547,62 @@
         <v>2026-09-04T11:41:47.445Z</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>30680aff-dffc-4170-9152-67ee539b3e93</v>
+      </c>
+      <c r="B11" t="str">
+        <v>e323d9c8-295f-472c-93f3-fefc39655d80</v>
+      </c>
+      <c r="C11" t="str">
+        <v>ปรับสีสถานะเพิ่มความเข็มขึ้น</v>
+      </c>
+      <c r="D11" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="E11" t="str">
+        <v>9</v>
+      </c>
+      <c r="F11" t="str">
+        <v>2026-09-11T06:55:08.648Z</v>
+      </c>
+      <c r="G11" t="str">
+        <v>2026-09-11T06:55:12.799Z</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>ba295d36-7862-4119-9b75-ab172c89a88e</v>
+      </c>
+      <c r="B12" t="str">
+        <v>e323d9c8-295f-472c-93f3-fefc39655d80</v>
+      </c>
+      <c r="C12" t="str">
+        <v>แก้ไขเงื่อนไขสรุปผลตรวจสุขภาพ</v>
+      </c>
+      <c r="D12" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="E12" t="str">
+        <v>10</v>
+      </c>
+      <c r="F12" t="str">
+        <v>2026-09-11T06:56:01.870Z</v>
+      </c>
+      <c r="G12" t="str">
+        <v>2026-09-11T06:56:01.870Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G12"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F36"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4067,110 +4706,110 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>b81e12b4-20a5-4fc4-a514-50370afcac96</v>
+        <v>76c55ffd-5c72-475c-9448-e969b036b7c0</v>
       </c>
       <c r="B6" t="str">
-        <v>1e95dc95-6f63-4810-9d57-8520eb9b42c5</v>
+        <v>e5a48211-b75f-4be3-aeee-dde8da731c1e</v>
       </c>
       <c r="C6" t="str">
-        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
       </c>
       <c r="D6" t="str">
         <v>0</v>
       </c>
       <c r="E6" t="str">
-        <v>2026-09-04T09:41:39.531Z</v>
+        <v>2026-09-04T09:47:39.835Z</v>
       </c>
       <c r="F6" t="str">
-        <v>2026-09-04T09:41:39.531Z</v>
+        <v>2026-09-04T09:47:39.835Z</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>76c55ffd-5c72-475c-9448-e969b036b7c0</v>
+        <v>689f964d-b216-40de-881b-605919cf6b35</v>
       </c>
       <c r="B7" t="str">
         <v>e5a48211-b75f-4be3-aeee-dde8da731c1e</v>
       </c>
       <c r="C7" t="str">
-        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
       <c r="D7" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E7" t="str">
-        <v>2026-09-04T09:47:39.835Z</v>
+        <v>2026-09-04T09:47:39.839Z</v>
       </c>
       <c r="F7" t="str">
-        <v>2026-09-04T09:47:39.835Z</v>
+        <v>2026-09-04T09:47:39.839Z</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>689f964d-b216-40de-881b-605919cf6b35</v>
+        <v>be30c4c5-9550-4b85-8401-c243a2cc9973</v>
       </c>
       <c r="B8" t="str">
-        <v>e5a48211-b75f-4be3-aeee-dde8da731c1e</v>
+        <v>2ee76ad4-4c3e-40be-9b97-9100e95fa1a7</v>
       </c>
       <c r="C8" t="str">
-        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
       </c>
       <c r="D8" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E8" t="str">
-        <v>2026-09-04T09:47:39.839Z</v>
+        <v>2026-09-04T09:48:58.065Z</v>
       </c>
       <c r="F8" t="str">
-        <v>2026-09-04T09:47:39.839Z</v>
+        <v>2026-09-04T09:48:58.065Z</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>be30c4c5-9550-4b85-8401-c243a2cc9973</v>
+        <v>6402d1cb-71a9-4249-9e8d-765a6d771490</v>
       </c>
       <c r="B9" t="str">
         <v>2ee76ad4-4c3e-40be-9b97-9100e95fa1a7</v>
       </c>
       <c r="C9" t="str">
-        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
+        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
       </c>
       <c r="D9" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" t="str">
-        <v>2026-09-04T09:48:58.065Z</v>
+        <v>2026-09-04T09:48:58.069Z</v>
       </c>
       <c r="F9" t="str">
-        <v>2026-09-04T09:48:58.065Z</v>
+        <v>2026-09-04T09:48:58.069Z</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>6402d1cb-71a9-4249-9e8d-765a6d771490</v>
+        <v>837b7f6d-8aa7-4477-a101-2bc781f457eb</v>
       </c>
       <c r="B10" t="str">
-        <v>2ee76ad4-4c3e-40be-9b97-9100e95fa1a7</v>
+        <v>e49e5c13-9c33-449b-9c2c-3b48f3119d16</v>
       </c>
       <c r="C10" t="str">
-        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
+        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
       </c>
       <c r="D10" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E10" t="str">
-        <v>2026-09-04T09:48:58.069Z</v>
+        <v>2026-09-04T10:15:31.431Z</v>
       </c>
       <c r="F10" t="str">
-        <v>2026-09-04T09:48:58.069Z</v>
+        <v>2026-09-04T10:15:31.431Z</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>837b7f6d-8aa7-4477-a101-2bc781f457eb</v>
+        <v>4e27d0ea-d725-4fd6-8af3-af70d286f196</v>
       </c>
       <c r="B11" t="str">
-        <v>e49e5c13-9c33-449b-9c2c-3b48f3119d16</v>
+        <v>81722c13-7a3f-4789-a1ac-a70c472369e0</v>
       </c>
       <c r="C11" t="str">
         <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
@@ -4179,58 +4818,58 @@
         <v>0</v>
       </c>
       <c r="E11" t="str">
-        <v>2026-09-04T10:15:31.431Z</v>
+        <v>2026-09-04T11:41:49.851Z</v>
       </c>
       <c r="F11" t="str">
-        <v>2026-09-04T10:15:31.431Z</v>
+        <v>2026-09-04T11:41:49.851Z</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>7bac2115-77f1-401f-ba0e-824e6d60f4fd</v>
+        <v>9c21d982-7ad7-4a32-8875-f8af532fdf47</v>
       </c>
       <c r="B12" t="str">
-        <v>e323d9c8-295f-472c-93f3-fefc39655d80</v>
+        <v>81722c13-7a3f-4789-a1ac-a70c472369e0</v>
       </c>
       <c r="C12" t="str">
-        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
       <c r="D12" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E12" t="str">
-        <v>2026-09-04T10:15:52.847Z</v>
+        <v>2026-09-04T11:41:49.858Z</v>
       </c>
       <c r="F12" t="str">
-        <v>2026-09-04T10:15:52.847Z</v>
+        <v>2026-09-04T11:41:49.858Z</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>4e27d0ea-d725-4fd6-8af3-af70d286f196</v>
+        <v>61cb483a-a74d-4d8f-b675-5383b14f8f77</v>
       </c>
       <c r="B13" t="str">
-        <v>81722c13-7a3f-4789-a1ac-a70c472369e0</v>
+        <v>efd54252-a5fb-4a92-ae20-141a96834757</v>
       </c>
       <c r="C13" t="str">
-        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
+        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
       </c>
       <c r="D13" t="str">
         <v>0</v>
       </c>
       <c r="E13" t="str">
-        <v>2026-09-04T11:41:49.851Z</v>
+        <v>2026-09-04T12:29:03.469Z</v>
       </c>
       <c r="F13" t="str">
-        <v>2026-09-04T11:41:49.851Z</v>
+        <v>2026-09-04T12:29:03.469Z</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>9c21d982-7ad7-4a32-8875-f8af532fdf47</v>
+        <v>fe14404c-70ae-4023-afd5-86198706c46a</v>
       </c>
       <c r="B14" t="str">
-        <v>81722c13-7a3f-4789-a1ac-a70c472369e0</v>
+        <v>efd54252-a5fb-4a92-ae20-141a96834757</v>
       </c>
       <c r="C14" t="str">
         <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
@@ -4239,18 +4878,18 @@
         <v>1</v>
       </c>
       <c r="E14" t="str">
-        <v>2026-09-04T11:41:49.858Z</v>
+        <v>2026-09-04T12:29:03.477Z</v>
       </c>
       <c r="F14" t="str">
-        <v>2026-09-04T11:41:49.858Z</v>
+        <v>2026-09-04T12:29:03.477Z</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>61cb483a-a74d-4d8f-b675-5383b14f8f77</v>
+        <v>5d381f35-c77e-4b8f-a9e7-4cbd4a8a52e8</v>
       </c>
       <c r="B15" t="str">
-        <v>efd54252-a5fb-4a92-ae20-141a96834757</v>
+        <v>b5647f0e-4c20-454b-b334-30c5458df783</v>
       </c>
       <c r="C15" t="str">
         <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
@@ -4259,18 +4898,18 @@
         <v>0</v>
       </c>
       <c r="E15" t="str">
-        <v>2026-09-04T12:29:03.469Z</v>
+        <v>2026-09-04T12:29:08.635Z</v>
       </c>
       <c r="F15" t="str">
-        <v>2026-09-04T12:29:03.469Z</v>
+        <v>2026-09-04T12:29:08.635Z</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>fe14404c-70ae-4023-afd5-86198706c46a</v>
+        <v>13efe219-b0c8-4dd9-82ca-e72d52723c88</v>
       </c>
       <c r="B16" t="str">
-        <v>efd54252-a5fb-4a92-ae20-141a96834757</v>
+        <v>b5647f0e-4c20-454b-b334-30c5458df783</v>
       </c>
       <c r="C16" t="str">
         <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
@@ -4279,38 +4918,38 @@
         <v>1</v>
       </c>
       <c r="E16" t="str">
-        <v>2026-09-04T12:29:03.477Z</v>
+        <v>2026-09-04T12:29:08.641Z</v>
       </c>
       <c r="F16" t="str">
-        <v>2026-09-04T12:29:03.477Z</v>
+        <v>2026-09-04T12:29:08.641Z</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>5d381f35-c77e-4b8f-a9e7-4cbd4a8a52e8</v>
+        <v>cff700c0-46bf-44de-83d8-60c73d4565d6</v>
       </c>
       <c r="B17" t="str">
-        <v>b5647f0e-4c20-454b-b334-30c5458df783</v>
+        <v>2982e690-f17b-4b39-8695-ca1ad2d39f5e</v>
       </c>
       <c r="C17" t="str">
-        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
+        <v>55d6e756-c40c-4755-84ab-c3458437acd6</v>
       </c>
       <c r="D17" t="str">
         <v>0</v>
       </c>
       <c r="E17" t="str">
-        <v>2026-09-04T12:29:08.635Z</v>
+        <v>2026-09-04T12:29:13.365Z</v>
       </c>
       <c r="F17" t="str">
-        <v>2026-09-04T12:29:08.635Z</v>
+        <v>2026-09-04T12:29:13.365Z</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>13efe219-b0c8-4dd9-82ca-e72d52723c88</v>
+        <v>db8acf76-4830-485d-9ee7-4300a8abc346</v>
       </c>
       <c r="B18" t="str">
-        <v>b5647f0e-4c20-454b-b334-30c5458df783</v>
+        <v>2982e690-f17b-4b39-8695-ca1ad2d39f5e</v>
       </c>
       <c r="C18" t="str">
         <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
@@ -4319,58 +4958,58 @@
         <v>1</v>
       </c>
       <c r="E18" t="str">
-        <v>2026-09-04T12:29:08.641Z</v>
+        <v>2026-09-04T12:29:13.371Z</v>
       </c>
       <c r="F18" t="str">
-        <v>2026-09-04T12:29:08.641Z</v>
+        <v>2026-09-04T12:29:13.371Z</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>cff700c0-46bf-44de-83d8-60c73d4565d6</v>
+        <v>a0bde16c-883f-435d-a1e6-3ff8173e27fc</v>
       </c>
       <c r="B19" t="str">
-        <v>2982e690-f17b-4b39-8695-ca1ad2d39f5e</v>
+        <v>b1e061e4-cef5-46b4-a149-31d4340bd038</v>
       </c>
       <c r="C19" t="str">
-        <v>55d6e756-c40c-4755-84ab-c3458437acd6</v>
+        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
       </c>
       <c r="D19" t="str">
         <v>0</v>
       </c>
       <c r="E19" t="str">
-        <v>2026-09-04T12:29:13.365Z</v>
+        <v>2026-09-04T12:29:18.501Z</v>
       </c>
       <c r="F19" t="str">
-        <v>2026-09-04T12:29:13.365Z</v>
+        <v>2026-09-04T12:29:18.501Z</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>db8acf76-4830-485d-9ee7-4300a8abc346</v>
+        <v>35763cf5-1687-4782-a94f-47223bc94f62</v>
       </c>
       <c r="B20" t="str">
-        <v>2982e690-f17b-4b39-8695-ca1ad2d39f5e</v>
+        <v>b1e061e4-cef5-46b4-a149-31d4340bd038</v>
       </c>
       <c r="C20" t="str">
-        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
       </c>
       <c r="D20" t="str">
         <v>1</v>
       </c>
       <c r="E20" t="str">
-        <v>2026-09-04T12:29:13.371Z</v>
+        <v>2026-09-04T12:29:18.507Z</v>
       </c>
       <c r="F20" t="str">
-        <v>2026-09-04T12:29:13.371Z</v>
+        <v>2026-09-04T12:29:18.507Z</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>a0bde16c-883f-435d-a1e6-3ff8173e27fc</v>
+        <v>035c1398-3263-4e99-8273-9aba0c9023ba</v>
       </c>
       <c r="B21" t="str">
-        <v>b1e061e4-cef5-46b4-a149-31d4340bd038</v>
+        <v>764fd6d8-3712-4019-8c67-6e3615085faf</v>
       </c>
       <c r="C21" t="str">
         <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
@@ -4379,18 +5018,18 @@
         <v>0</v>
       </c>
       <c r="E21" t="str">
-        <v>2026-09-04T12:29:18.501Z</v>
+        <v>2026-09-04T12:29:22.908Z</v>
       </c>
       <c r="F21" t="str">
-        <v>2026-09-04T12:29:18.501Z</v>
+        <v>2026-09-04T12:29:22.908Z</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>35763cf5-1687-4782-a94f-47223bc94f62</v>
+        <v>544f63ce-d992-4c80-aaac-33a8fa860614</v>
       </c>
       <c r="B22" t="str">
-        <v>b1e061e4-cef5-46b4-a149-31d4340bd038</v>
+        <v>764fd6d8-3712-4019-8c67-6e3615085faf</v>
       </c>
       <c r="C22" t="str">
         <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
@@ -4399,158 +5038,158 @@
         <v>1</v>
       </c>
       <c r="E22" t="str">
-        <v>2026-09-04T12:29:18.507Z</v>
+        <v>2026-09-04T12:29:22.912Z</v>
       </c>
       <c r="F22" t="str">
-        <v>2026-09-04T12:29:18.507Z</v>
+        <v>2026-09-04T12:29:22.912Z</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>035c1398-3263-4e99-8273-9aba0c9023ba</v>
+        <v>5da43984-fa10-419d-be97-55c04f991d54</v>
       </c>
       <c r="B23" t="str">
-        <v>764fd6d8-3712-4019-8c67-6e3615085faf</v>
+        <v>d6acd7ea-e69f-4894-9ce4-c8ae86da6bd2</v>
       </c>
       <c r="C23" t="str">
-        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
+        <v>55d6e756-c40c-4755-84ab-c3458437acd6</v>
       </c>
       <c r="D23" t="str">
         <v>0</v>
       </c>
       <c r="E23" t="str">
-        <v>2026-09-04T12:29:22.908Z</v>
+        <v>2026-09-04T12:29:28.748Z</v>
       </c>
       <c r="F23" t="str">
-        <v>2026-09-04T12:29:22.908Z</v>
+        <v>2026-09-04T12:29:28.748Z</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>544f63ce-d992-4c80-aaac-33a8fa860614</v>
+        <v>9c43d17e-fee0-4a90-b4b0-7076e3a5fda9</v>
       </c>
       <c r="B24" t="str">
-        <v>764fd6d8-3712-4019-8c67-6e3615085faf</v>
+        <v>a4db697d-4d50-4200-8355-647ab86cd480</v>
       </c>
       <c r="C24" t="str">
-        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
+        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
       </c>
       <c r="D24" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E24" t="str">
-        <v>2026-09-04T12:29:22.912Z</v>
+        <v>2026-09-08T02:27:47.879Z</v>
       </c>
       <c r="F24" t="str">
-        <v>2026-09-04T12:29:22.912Z</v>
+        <v>2026-09-08T02:27:47.879Z</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>5da43984-fa10-419d-be97-55c04f991d54</v>
+        <v>2c1e3965-52ed-4324-98bc-d48def9e2254</v>
       </c>
       <c r="B25" t="str">
-        <v>d6acd7ea-e69f-4894-9ce4-c8ae86da6bd2</v>
+        <v>a4db697d-4d50-4200-8355-647ab86cd480</v>
       </c>
       <c r="C25" t="str">
-        <v>55d6e756-c40c-4755-84ab-c3458437acd6</v>
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
       <c r="D25" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E25" t="str">
-        <v>2026-09-04T12:29:28.748Z</v>
+        <v>2026-09-08T02:27:47.888Z</v>
       </c>
       <c r="F25" t="str">
-        <v>2026-09-04T12:29:28.748Z</v>
+        <v>2026-09-08T02:27:47.888Z</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>9c43d17e-fee0-4a90-b4b0-7076e3a5fda9</v>
+        <v>b3b7233e-4aaf-4596-aa01-e044607b2861</v>
       </c>
       <c r="B26" t="str">
-        <v>a4db697d-4d50-4200-8355-647ab86cd480</v>
+        <v>12f8c884-7a9e-4086-8352-ace2ea778248</v>
       </c>
       <c r="C26" t="str">
-        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
+        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
       </c>
       <c r="D26" t="str">
         <v>0</v>
       </c>
       <c r="E26" t="str">
-        <v>2026-09-08T02:27:47.879Z</v>
+        <v>2026-09-08T03:13:32.577Z</v>
       </c>
       <c r="F26" t="str">
-        <v>2026-09-08T02:27:47.879Z</v>
+        <v>2026-09-08T03:13:32.577Z</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>2c1e3965-52ed-4324-98bc-d48def9e2254</v>
+        <v>ba8ae40b-58f0-4048-a945-af20bbc3f415</v>
       </c>
       <c r="B27" t="str">
-        <v>a4db697d-4d50-4200-8355-647ab86cd480</v>
+        <v>58f112bb-1a6e-4e26-8d8a-9bcd3e5bc31d</v>
       </c>
       <c r="C27" t="str">
-        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
       </c>
       <c r="D27" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E27" t="str">
-        <v>2026-09-08T02:27:47.888Z</v>
+        <v>2026-09-08T07:00:38.362Z</v>
       </c>
       <c r="F27" t="str">
-        <v>2026-09-08T02:27:47.888Z</v>
+        <v>2026-09-08T07:00:38.362Z</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>2030cc27-64e7-4348-a193-88c452d06ec4</v>
+        <v>49b20734-492a-4950-9f99-ef820a888dc0</v>
       </c>
       <c r="B28" t="str">
-        <v>6ac09b86-b7ee-4b62-b048-4594eca71b6c</v>
+        <v>58f112bb-1a6e-4e26-8d8a-9bcd3e5bc31d</v>
       </c>
       <c r="C28" t="str">
-        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
       <c r="D28" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E28" t="str">
-        <v>2026-09-08T03:12:47.728Z</v>
+        <v>2026-09-08T07:00:38.372Z</v>
       </c>
       <c r="F28" t="str">
-        <v>2026-09-08T03:12:47.728Z</v>
+        <v>2026-09-08T07:00:38.372Z</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>b3b7233e-4aaf-4596-aa01-e044607b2861</v>
+        <v>20bd867f-f75b-4d0b-8041-ab6406c30788</v>
       </c>
       <c r="B29" t="str">
-        <v>12f8c884-7a9e-4086-8352-ace2ea778248</v>
+        <v>c1b2bc1d-f4c5-42ea-bdc8-4fdc41bfd8ee</v>
       </c>
       <c r="C29" t="str">
-        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
       <c r="D29" t="str">
         <v>0</v>
       </c>
       <c r="E29" t="str">
-        <v>2026-09-08T03:13:32.577Z</v>
+        <v>2026-09-11T06:48:04.034Z</v>
       </c>
       <c r="F29" t="str">
-        <v>2026-09-08T03:13:32.577Z</v>
+        <v>2026-09-11T06:48:04.034Z</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>ba8ae40b-58f0-4048-a945-af20bbc3f415</v>
+        <v>9858a349-bd2a-4b33-99a3-dcd1a4e0023c</v>
       </c>
       <c r="B30" t="str">
-        <v>58f112bb-1a6e-4e26-8d8a-9bcd3e5bc31d</v>
+        <v>576fbffe-152c-4052-834c-1d230af3784a</v>
       </c>
       <c r="C30" t="str">
         <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
@@ -4559,18 +5198,18 @@
         <v>0</v>
       </c>
       <c r="E30" t="str">
-        <v>2026-09-08T07:00:38.362Z</v>
+        <v>2026-09-11T06:48:10.741Z</v>
       </c>
       <c r="F30" t="str">
-        <v>2026-09-08T07:00:38.362Z</v>
+        <v>2026-09-11T06:48:10.741Z</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>49b20734-492a-4950-9f99-ef820a888dc0</v>
+        <v>a491ec90-2d22-49e2-832d-a5c7e77f3802</v>
       </c>
       <c r="B31" t="str">
-        <v>58f112bb-1a6e-4e26-8d8a-9bcd3e5bc31d</v>
+        <v>576fbffe-152c-4052-834c-1d230af3784a</v>
       </c>
       <c r="C31" t="str">
         <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
@@ -4579,38 +5218,38 @@
         <v>1</v>
       </c>
       <c r="E31" t="str">
-        <v>2026-09-08T07:00:38.372Z</v>
+        <v>2026-09-11T06:48:10.757Z</v>
       </c>
       <c r="F31" t="str">
-        <v>2026-09-08T07:00:38.372Z</v>
+        <v>2026-09-11T06:48:10.757Z</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>dee4af21-e9a1-40ae-b72a-dcbf02909835</v>
+        <v>de6dc226-235c-4da0-a30f-e75d4aca61e5</v>
       </c>
       <c r="B32" t="str">
-        <v>576fbffe-152c-4052-834c-1d230af3784a</v>
+        <v>a2d08247-d1c8-4c29-9663-96adb51418ff</v>
       </c>
       <c r="C32" t="str">
-        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
+        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
       </c>
       <c r="D32" t="str">
         <v>0</v>
       </c>
       <c r="E32" t="str">
-        <v>2026-09-08T07:00:51.130Z</v>
+        <v>2026-09-11T06:49:21.285Z</v>
       </c>
       <c r="F32" t="str">
-        <v>2026-09-08T07:00:51.130Z</v>
+        <v>2026-09-11T06:49:21.285Z</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>9caf7a0a-46c6-4476-b1df-0b18e5e53d52</v>
+        <v>d99f05b1-5193-452c-b1ac-afbc759d8cac</v>
       </c>
       <c r="B33" t="str">
-        <v>576fbffe-152c-4052-834c-1d230af3784a</v>
+        <v>a2d08247-d1c8-4c29-9663-96adb51418ff</v>
       </c>
       <c r="C33" t="str">
         <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
@@ -4619,18 +5258,18 @@
         <v>1</v>
       </c>
       <c r="E33" t="str">
-        <v>2026-09-08T07:00:51.140Z</v>
+        <v>2026-09-11T06:49:21.297Z</v>
       </c>
       <c r="F33" t="str">
-        <v>2026-09-08T07:00:51.140Z</v>
+        <v>2026-09-11T06:49:21.297Z</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>ca84d7b2-4097-412c-a221-df5574d728c3</v>
+        <v>260bb430-4d1d-4d94-933e-83126ec77f7c</v>
       </c>
       <c r="B34" t="str">
-        <v>c1b2bc1d-f4c5-42ea-bdc8-4fdc41bfd8ee</v>
+        <v>1e95dc95-6f63-4810-9d57-8520eb9b42c5</v>
       </c>
       <c r="C34" t="str">
         <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
@@ -4639,15 +5278,55 @@
         <v>0</v>
       </c>
       <c r="E34" t="str">
-        <v>2026-09-08T07:22:32.129Z</v>
+        <v>2026-09-11T06:49:45.495Z</v>
       </c>
       <c r="F34" t="str">
-        <v>2026-09-08T07:22:32.129Z</v>
+        <v>2026-09-11T06:49:45.495Z</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>5f14d6ba-83fa-45f2-b869-5981498a8b3a</v>
+      </c>
+      <c r="B35" t="str">
+        <v>e323d9c8-295f-472c-93f3-fefc39655d80</v>
+      </c>
+      <c r="C35" t="str">
+        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
+      </c>
+      <c r="D35" t="str">
+        <v>0</v>
+      </c>
+      <c r="E35" t="str">
+        <v>2026-09-11T06:56:21.627Z</v>
+      </c>
+      <c r="F35" t="str">
+        <v>2026-09-11T06:56:21.627Z</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>96cc8b37-e673-419a-bf8d-08393ece27ae</v>
+      </c>
+      <c r="B36" t="str">
+        <v>6ac09b86-b7ee-4b62-b048-4594eca71b6c</v>
+      </c>
+      <c r="C36" t="str">
+        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
+      </c>
+      <c r="D36" t="str">
+        <v>0</v>
+      </c>
+      <c r="E36" t="str">
+        <v>2026-09-11T06:58:59.731Z</v>
+      </c>
+      <c r="F36" t="str">
+        <v>2026-09-11T06:58:59.731Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F34"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F36"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: introduce tagging system for tasks
- Added a new TagOption model to the database schema for managing task tags.
- Updated task model to include a tags field, allowing tasks to be associated with multiple tags.
- Implemented tag management in the settings dialog, enabling users to add, edit, and delete tags.
- Enhanced task forms and views to support tag selection and display, improving task tracking.
- Updated taskDB.xlsx to reflect changes in task and tag structures.
</commit_message>
<xml_diff>
--- a/data/taskDB.xlsx
+++ b/data/taskDB.xlsx
@@ -13,6 +13,7 @@
     <sheet name="TaskAssignees" sheetId="8" r:id="rId8"/>
     <sheet name="TaskTypes" sheetId="9" r:id="rId9"/>
     <sheet name="SubtaskAssignees" sheetId="10" r:id="rId10"/>
+    <sheet name="Tags" sheetId="11" r:id="rId11"/>
   </sheets>
 </workbook>
 </file>
@@ -406,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -454,16 +455,62 @@
         <v>2026-09-08T07:06:14.659Z</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>1eb871dc-ccd4-4308-93fb-d7ce7c5fc3dd</v>
+      </c>
+      <c r="B3" t="str">
+        <v>FWF Approve Claim</v>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v>#22C55E</v>
+      </c>
+      <c r="E3" t="str">
+        <v>1</v>
+      </c>
+      <c r="F3" t="str">
+        <v>2026-09-11T09:32:13.972Z</v>
+      </c>
+      <c r="G3" t="str">
+        <v>2026-09-11T09:32:13.972Z</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>277790ac-fdb8-4cfa-a383-11aebb2976fc</v>
+      </c>
+      <c r="B4" t="str">
+        <v>FHD</v>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v>#6BB82A</v>
+      </c>
+      <c r="E4" t="str">
+        <v>2</v>
+      </c>
+      <c r="F4" t="str">
+        <v>2026-09-11T09:32:22.454Z</v>
+      </c>
+      <c r="G4" t="str">
+        <v>2026-09-11T09:32:22.454Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -587,10 +634,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>d47d2637-7aee-4c15-9f28-7db15c5d735b</v>
+        <v>888a6d5c-c169-4644-ad30-0aa6b9d3048a</v>
       </c>
       <c r="B7" t="str">
-        <v>e5435e0d-9a20-4241-adc6-e880dc6bd3d2</v>
+        <v>c9699cc1-1683-4feb-984e-878d32682885</v>
       </c>
       <c r="C7" t="str">
         <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
@@ -599,18 +646,18 @@
         <v>0</v>
       </c>
       <c r="E7" t="str">
-        <v>2026-09-04T10:15:49.861Z</v>
+        <v>2026-09-04T10:15:50.569Z</v>
       </c>
       <c r="F7" t="str">
-        <v>2026-09-04T10:15:49.861Z</v>
+        <v>2026-09-04T10:15:50.569Z</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>888a6d5c-c169-4644-ad30-0aa6b9d3048a</v>
+        <v>1a7cd58c-3775-46bf-8b3b-0793b1e36035</v>
       </c>
       <c r="B8" t="str">
-        <v>c9699cc1-1683-4feb-984e-878d32682885</v>
+        <v>4657d602-61e3-4999-8fd6-2b2eda534e20</v>
       </c>
       <c r="C8" t="str">
         <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
@@ -619,95 +666,266 @@
         <v>0</v>
       </c>
       <c r="E8" t="str">
-        <v>2026-09-04T10:15:50.569Z</v>
+        <v>2026-09-04T10:15:51.162Z</v>
       </c>
       <c r="F8" t="str">
-        <v>2026-09-04T10:15:50.569Z</v>
+        <v>2026-09-04T10:15:51.162Z</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>1a7cd58c-3775-46bf-8b3b-0793b1e36035</v>
+        <v>3f02a3c6-4846-489a-8ad3-8add2bd12235</v>
       </c>
       <c r="B9" t="str">
-        <v>4657d602-61e3-4999-8fd6-2b2eda534e20</v>
+        <v>d3abd120-8ba6-4dca-b36e-64c8291bcc93</v>
       </c>
       <c r="C9" t="str">
-        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
       <c r="D9" t="str">
         <v>0</v>
       </c>
       <c r="E9" t="str">
-        <v>2026-09-04T10:15:51.162Z</v>
+        <v>2026-09-04T11:41:47.465Z</v>
       </c>
       <c r="F9" t="str">
-        <v>2026-09-04T10:15:51.162Z</v>
+        <v>2026-09-04T11:41:47.465Z</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>3f02a3c6-4846-489a-8ad3-8add2bd12235</v>
+        <v>ee8bf0b0-933f-475c-a471-0ddfb283a833</v>
       </c>
       <c r="B10" t="str">
-        <v>d3abd120-8ba6-4dca-b36e-64c8291bcc93</v>
+        <v>ba295d36-7862-4119-9b75-ab172c89a88e</v>
       </c>
       <c r="C10" t="str">
-        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
       </c>
       <c r="D10" t="str">
         <v>0</v>
       </c>
       <c r="E10" t="str">
-        <v>2026-09-04T11:41:47.465Z</v>
+        <v>2026-09-11T06:56:01.912Z</v>
       </c>
       <c r="F10" t="str">
-        <v>2026-09-04T11:41:47.465Z</v>
+        <v>2026-09-11T06:56:01.912Z</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>18a4faac-4efd-4b46-ac5b-1888d942a675</v>
+        <v>7c5f731a-53a8-43c3-825a-ef7efbb9d822</v>
       </c>
       <c r="B11" t="str">
-        <v>30680aff-dffc-4170-9152-67ee539b3e93</v>
+        <v>bfe255cd-98bd-40a3-96e1-ab996fe7202c</v>
       </c>
       <c r="C11" t="str">
-        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
       <c r="D11" t="str">
         <v>0</v>
       </c>
       <c r="E11" t="str">
-        <v>2026-09-11T06:55:12.829Z</v>
+        <v>2026-09-11T08:17:31.140Z</v>
       </c>
       <c r="F11" t="str">
-        <v>2026-09-11T06:55:12.829Z</v>
+        <v>2026-09-11T08:17:31.140Z</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>ee8bf0b0-933f-475c-a471-0ddfb283a833</v>
+        <v>ce82216d-6f40-419b-8ebc-7112bbe25e5f</v>
       </c>
       <c r="B12" t="str">
-        <v>ba295d36-7862-4119-9b75-ab172c89a88e</v>
+        <v>f17a5ff5-5c29-4c90-a446-189127086d64</v>
       </c>
       <c r="C12" t="str">
-        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
       <c r="D12" t="str">
         <v>0</v>
       </c>
       <c r="E12" t="str">
-        <v>2026-09-11T06:56:01.912Z</v>
+        <v>2026-09-11T08:17:32.876Z</v>
       </c>
       <c r="F12" t="str">
-        <v>2026-09-11T06:56:01.912Z</v>
+        <v>2026-09-11T08:17:32.876Z</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>9863b512-060a-4f96-8ad2-3cb08a8b7d91</v>
+      </c>
+      <c r="B13" t="str">
+        <v>4edb6864-2622-4350-b92b-c0c48bbb8deb</v>
+      </c>
+      <c r="C13" t="str">
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+      </c>
+      <c r="D13" t="str">
+        <v>0</v>
+      </c>
+      <c r="E13" t="str">
+        <v>2026-09-11T08:17:33.495Z</v>
+      </c>
+      <c r="F13" t="str">
+        <v>2026-09-11T08:17:33.495Z</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>53f816cc-9fc5-4a46-9785-aeb85a874765</v>
+      </c>
+      <c r="B14" t="str">
+        <v>65a8c469-13cb-4029-84bb-d97fbfe839b5</v>
+      </c>
+      <c r="C14" t="str">
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+      </c>
+      <c r="D14" t="str">
+        <v>0</v>
+      </c>
+      <c r="E14" t="str">
+        <v>2026-09-11T08:17:34.271Z</v>
+      </c>
+      <c r="F14" t="str">
+        <v>2026-09-11T08:17:34.271Z</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>84d8dc7a-e9e9-4f79-a69e-798ccbb0f734</v>
+      </c>
+      <c r="B15" t="str">
+        <v>425ff6e2-40e5-41fd-bb1a-ef0a523ee4c5</v>
+      </c>
+      <c r="C15" t="str">
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+      </c>
+      <c r="D15" t="str">
+        <v>0</v>
+      </c>
+      <c r="E15" t="str">
+        <v>2026-09-11T08:17:34.812Z</v>
+      </c>
+      <c r="F15" t="str">
+        <v>2026-09-11T08:17:34.812Z</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>6afebc55-e1d0-4966-a2a2-b1352edf7ef5</v>
+      </c>
+      <c r="B16" t="str">
+        <v>c577077b-27fa-405a-b8f9-50fb7f3f2550</v>
+      </c>
+      <c r="C16" t="str">
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+      </c>
+      <c r="D16" t="str">
+        <v>0</v>
+      </c>
+      <c r="E16" t="str">
+        <v>2026-09-11T08:17:36.056Z</v>
+      </c>
+      <c r="F16" t="str">
+        <v>2026-09-11T08:17:36.056Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F16"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F4"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>name</v>
+      </c>
+      <c r="C1" t="str">
+        <v>color</v>
+      </c>
+      <c r="D1" t="str">
+        <v>sortOrder</v>
+      </c>
+      <c r="E1" t="str">
+        <v>createdAt</v>
+      </c>
+      <c r="F1" t="str">
+        <v>updatedAt</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>f30a626b-0955-400f-8972-0336e1abf8bc</v>
+      </c>
+      <c r="B2" t="str">
+        <v>บัค</v>
+      </c>
+      <c r="C2" t="str">
+        <v>#EF4444</v>
+      </c>
+      <c r="D2" t="str">
+        <v>0</v>
+      </c>
+      <c r="E2" t="str">
+        <v>2026-09-11T10:23:50.233Z</v>
+      </c>
+      <c r="F2" t="str">
+        <v>2026-09-11T10:23:50.233Z</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>072757fe-2fe3-4341-a3b9-a288d4e4026d</v>
+      </c>
+      <c r="B3" t="str">
+        <v>ปรับเพิ่ม</v>
+      </c>
+      <c r="C3" t="str">
+        <v>#F97316</v>
+      </c>
+      <c r="D3" t="str">
+        <v>1</v>
+      </c>
+      <c r="E3" t="str">
+        <v>2026-09-11T10:23:50.251Z</v>
+      </c>
+      <c r="F3" t="str">
+        <v>2026-09-11T10:23:50.251Z</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>91a615d0-bb29-4c26-8677-700da86017fa</v>
+      </c>
+      <c r="B4" t="str">
+        <v>วิธีการเพิ่มเติม</v>
+      </c>
+      <c r="C4" t="str">
+        <v>#8B5CF6</v>
+      </c>
+      <c r="D4" t="str">
+        <v>2</v>
+      </c>
+      <c r="E4" t="str">
+        <v>2026-09-11T10:23:50.269Z</v>
+      </c>
+      <c r="F4" t="str">
+        <v>2026-09-11T10:23:50.269Z</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -805,7 +1023,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -844,7 +1062,7 @@
         <v>2026-09-01T07:23:24.979Z</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-09-11T07:10:49.660Z</v>
+        <v>2026-09-11T10:29:36.079Z</v>
       </c>
     </row>
     <row r="3">
@@ -864,7 +1082,7 @@
         <v>2026-09-01T07:23:24.981Z</v>
       </c>
       <c r="F3" t="str">
-        <v>2026-09-11T07:10:49.664Z</v>
+        <v>2026-09-11T10:29:36.084Z</v>
       </c>
     </row>
     <row r="4">
@@ -884,7 +1102,7 @@
         <v>2026-09-01T07:23:24.983Z</v>
       </c>
       <c r="F4" t="str">
-        <v>2026-09-11T07:10:49.671Z</v>
+        <v>2026-09-11T10:29:36.095Z</v>
       </c>
     </row>
     <row r="5">
@@ -904,7 +1122,7 @@
         <v>2026-09-01T07:23:24.985Z</v>
       </c>
       <c r="F5" t="str">
-        <v>2026-09-11T07:10:49.667Z</v>
+        <v>2026-09-11T10:29:36.090Z</v>
       </c>
     </row>
     <row r="6">
@@ -924,32 +1142,12 @@
         <v>2026-09-01T07:23:24.988Z</v>
       </c>
       <c r="F6" t="str">
-        <v>2026-09-11T07:10:49.675Z</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>f568698e-99c5-418d-8036-5f99072d6e28</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Fixing</v>
-      </c>
-      <c r="C7" t="str">
-        <v>#F7D83B</v>
-      </c>
-      <c r="D7" t="str">
-        <v>2</v>
-      </c>
-      <c r="E7" t="str">
-        <v>2026-09-11T06:54:30.253Z</v>
-      </c>
-      <c r="F7" t="str">
-        <v>2026-09-11T06:54:36.730Z</v>
+        <v>2026-09-11T10:29:36.099Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F6"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1255,7 +1453,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q25"/>
+  <dimension ref="A1:R34"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1274,39 +1472,42 @@
         <v>taskType</v>
       </c>
       <c r="F1" t="str">
+        <v>tags</v>
+      </c>
+      <c r="G1" t="str">
         <v>startDate</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>endDate</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>uatDate</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>prdDate</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>sortOrder</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>projectId</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>priorityId</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>statusId</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>assigneeId</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>ownerId</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
         <v>createdAt</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="R1" t="str">
         <v>updatedAt</v>
       </c>
     </row>
@@ -1327,39 +1528,42 @@
         <v>Back End</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-08-31</v>
+        <v/>
       </c>
       <c r="G2" t="str">
         <v>2026-08-31</v>
       </c>
       <c r="H2" t="str">
-        <v/>
+        <v>2026-08-31</v>
       </c>
       <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
         <v>2026-08-31</v>
       </c>
-      <c r="J2" t="str">
-        <v>0</v>
-      </c>
       <c r="K2" t="str">
+        <v>0</v>
+      </c>
+      <c r="L2" t="str">
         <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
       </c>
-      <c r="L2" t="str">
+      <c r="M2" t="str">
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
-      <c r="M2" t="str">
+      <c r="N2" t="str">
         <v>e475d16a-9163-4793-b90e-9aed0ce0e9ec</v>
       </c>
-      <c r="N2" t="str">
+      <c r="O2" t="str">
         <v>55d6e756-c40c-4755-84ab-c3458437acd6</v>
       </c>
-      <c r="O2" t="str">
-        <v/>
-      </c>
       <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
         <v>2026-09-04T09:22:21.943Z</v>
       </c>
-      <c r="Q2" t="str">
+      <c r="R2" t="str">
         <v>2026-09-04T12:29:28.753Z</v>
       </c>
     </row>
@@ -1380,39 +1584,42 @@
         <v>Back End, Front End</v>
       </c>
       <c r="F3" t="str">
-        <v>2026-08-31</v>
+        <v/>
       </c>
       <c r="G3" t="str">
         <v>2026-08-31</v>
       </c>
       <c r="H3" t="str">
-        <v/>
+        <v>2026-08-31</v>
       </c>
       <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
         <v>2026-08-31</v>
       </c>
-      <c r="J3" t="str">
-        <v>0</v>
-      </c>
       <c r="K3" t="str">
+        <v>0</v>
+      </c>
+      <c r="L3" t="str">
         <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
       </c>
-      <c r="L3" t="str">
+      <c r="M3" t="str">
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
-      <c r="M3" t="str">
+      <c r="N3" t="str">
         <v>e475d16a-9163-4793-b90e-9aed0ce0e9ec</v>
       </c>
-      <c r="N3" t="str">
+      <c r="O3" t="str">
         <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
       </c>
-      <c r="O3" t="str">
-        <v/>
-      </c>
       <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
         <v>2026-09-04T09:24:04.693Z</v>
       </c>
-      <c r="Q3" t="str">
+      <c r="R3" t="str">
         <v>2026-09-04T12:29:22.917Z</v>
       </c>
     </row>
@@ -1433,39 +1640,42 @@
         <v>Back End, Front End</v>
       </c>
       <c r="F4" t="str">
-        <v>2026-08-31</v>
+        <v/>
       </c>
       <c r="G4" t="str">
         <v>2026-08-31</v>
       </c>
       <c r="H4" t="str">
-        <v/>
+        <v>2026-08-31</v>
       </c>
       <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
         <v>2026-08-31</v>
       </c>
-      <c r="J4" t="str">
-        <v>0</v>
-      </c>
       <c r="K4" t="str">
+        <v>0</v>
+      </c>
+      <c r="L4" t="str">
         <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
       </c>
-      <c r="L4" t="str">
+      <c r="M4" t="str">
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
-      <c r="M4" t="str">
+      <c r="N4" t="str">
         <v>e475d16a-9163-4793-b90e-9aed0ce0e9ec</v>
       </c>
-      <c r="N4" t="str">
+      <c r="O4" t="str">
         <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
       </c>
-      <c r="O4" t="str">
-        <v/>
-      </c>
       <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
         <v>2026-09-04T09:24:33.365Z</v>
       </c>
-      <c r="Q4" t="str">
+      <c r="R4" t="str">
         <v>2026-09-04T12:29:18.513Z</v>
       </c>
     </row>
@@ -1486,39 +1696,42 @@
         <v>Back End</v>
       </c>
       <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
         <v>2026-08-31</v>
       </c>
-      <c r="G5" t="str">
+      <c r="H5" t="str">
         <v>2026-09-01</v>
       </c>
-      <c r="H5" t="str">
-        <v/>
-      </c>
       <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
         <v>2026-09-01</v>
       </c>
-      <c r="J5" t="str">
-        <v>0</v>
-      </c>
       <c r="K5" t="str">
+        <v>0</v>
+      </c>
+      <c r="L5" t="str">
         <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
       </c>
-      <c r="L5" t="str">
+      <c r="M5" t="str">
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
-      <c r="M5" t="str">
+      <c r="N5" t="str">
         <v>e475d16a-9163-4793-b90e-9aed0ce0e9ec</v>
       </c>
-      <c r="N5" t="str">
+      <c r="O5" t="str">
         <v>55d6e756-c40c-4755-84ab-c3458437acd6</v>
       </c>
-      <c r="O5" t="str">
-        <v/>
-      </c>
       <c r="P5" t="str">
+        <v/>
+      </c>
+      <c r="Q5" t="str">
         <v>2026-09-04T09:25:10.002Z</v>
       </c>
-      <c r="Q5" t="str">
+      <c r="R5" t="str">
         <v>2026-09-04T12:29:13.377Z</v>
       </c>
     </row>
@@ -1539,10 +1752,10 @@
         <v>Back End, Front End</v>
       </c>
       <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
         <v>2026-08-31</v>
-      </c>
-      <c r="G6" t="str">
-        <v>2026-09-02</v>
       </c>
       <c r="H6" t="str">
         <v>2026-09-02</v>
@@ -1551,27 +1764,30 @@
         <v>2026-09-02</v>
       </c>
       <c r="J6" t="str">
-        <v>0</v>
+        <v>2026-09-02</v>
       </c>
       <c r="K6" t="str">
+        <v>0</v>
+      </c>
+      <c r="L6" t="str">
         <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
       </c>
-      <c r="L6" t="str">
+      <c r="M6" t="str">
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
-      <c r="M6" t="str">
+      <c r="N6" t="str">
         <v>e475d16a-9163-4793-b90e-9aed0ce0e9ec</v>
       </c>
-      <c r="N6" t="str">
+      <c r="O6" t="str">
         <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
       </c>
-      <c r="O6" t="str">
-        <v/>
-      </c>
       <c r="P6" t="str">
+        <v/>
+      </c>
+      <c r="Q6" t="str">
         <v>2026-09-04T09:26:00.676Z</v>
       </c>
-      <c r="Q6" t="str">
+      <c r="R6" t="str">
         <v>2026-09-04T12:29:08.647Z</v>
       </c>
     </row>
@@ -1592,40 +1808,43 @@
         <v>Front End</v>
       </c>
       <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
         <v>2026-08-31</v>
       </c>
-      <c r="G7" t="str">
+      <c r="H7" t="str">
         <v>2026-09-04</v>
       </c>
-      <c r="H7" t="str">
+      <c r="I7" t="str">
         <v>2026-09-14</v>
       </c>
-      <c r="I7" t="str">
+      <c r="J7" t="str">
         <v>2026-09-16</v>
       </c>
-      <c r="J7" t="str">
-        <v>0</v>
-      </c>
       <c r="K7" t="str">
+        <v>0</v>
+      </c>
+      <c r="L7" t="str">
         <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
       </c>
-      <c r="L7" t="str">
+      <c r="M7" t="str">
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
-      <c r="M7" t="str">
-        <v>f568698e-99c5-418d-8036-5f99072d6e28</v>
-      </c>
       <c r="N7" t="str">
+        <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
+      </c>
+      <c r="O7" t="str">
         <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
       </c>
-      <c r="O7" t="str">
-        <v/>
-      </c>
       <c r="P7" t="str">
+        <v/>
+      </c>
+      <c r="Q7" t="str">
         <v>2026-09-04T09:27:00.612Z</v>
       </c>
-      <c r="Q7" t="str">
-        <v>2026-09-11T06:56:21.637Z</v>
+      <c r="R7" t="str">
+        <v>2026-09-11T09:28:49.738Z</v>
       </c>
     </row>
     <row r="8">
@@ -1645,39 +1864,42 @@
         <v>Back End</v>
       </c>
       <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
         <v>2026-08-31</v>
       </c>
-      <c r="G8" t="str">
+      <c r="H8" t="str">
         <v>2026-09-04</v>
       </c>
-      <c r="H8" t="str">
+      <c r="I8" t="str">
         <v>2026-09-02</v>
       </c>
-      <c r="I8" t="str">
+      <c r="J8" t="str">
         <v>2026-09-13</v>
       </c>
-      <c r="J8" t="str">
-        <v>0</v>
-      </c>
       <c r="K8" t="str">
+        <v>0</v>
+      </c>
+      <c r="L8" t="str">
         <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
       </c>
-      <c r="L8" t="str">
+      <c r="M8" t="str">
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
-      <c r="M8" t="str">
+      <c r="N8" t="str">
         <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
       </c>
-      <c r="N8" t="str">
+      <c r="O8" t="str">
         <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
-      <c r="O8" t="str">
-        <v/>
-      </c>
       <c r="P8" t="str">
+        <v/>
+      </c>
+      <c r="Q8" t="str">
         <v>2026-09-04T09:29:47.993Z</v>
       </c>
-      <c r="Q8" t="str">
+      <c r="R8" t="str">
         <v>2026-09-11T06:49:45.510Z</v>
       </c>
     </row>
@@ -1698,39 +1920,42 @@
         <v>Back End, Front End</v>
       </c>
       <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
         <v>2026-08-31</v>
       </c>
-      <c r="G9" t="str">
+      <c r="H9" t="str">
         <v>2026-09-02</v>
       </c>
-      <c r="H9" t="str">
-        <v/>
-      </c>
       <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
         <v>2026-09-02</v>
       </c>
-      <c r="J9" t="str">
-        <v>0</v>
-      </c>
       <c r="K9" t="str">
+        <v>0</v>
+      </c>
+      <c r="L9" t="str">
         <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
       </c>
-      <c r="L9" t="str">
+      <c r="M9" t="str">
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
-      <c r="M9" t="str">
+      <c r="N9" t="str">
         <v>e475d16a-9163-4793-b90e-9aed0ce0e9ec</v>
       </c>
-      <c r="N9" t="str">
+      <c r="O9" t="str">
         <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
       </c>
-      <c r="O9" t="str">
-        <v/>
-      </c>
       <c r="P9" t="str">
+        <v/>
+      </c>
+      <c r="Q9" t="str">
         <v>2026-09-04T09:32:18.156Z</v>
       </c>
-      <c r="Q9" t="str">
+      <c r="R9" t="str">
         <v>2026-09-04T12:29:03.482Z</v>
       </c>
     </row>
@@ -1751,39 +1976,42 @@
         <v>Back End, Front End</v>
       </c>
       <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10" t="str">
         <v>2026-08-31</v>
-      </c>
-      <c r="G10" t="str">
-        <v>2026-09-04</v>
       </c>
       <c r="H10" t="str">
         <v>2026-09-04</v>
       </c>
       <c r="I10" t="str">
-        <v/>
+        <v>2026-09-04</v>
       </c>
       <c r="J10" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="K10" t="str">
+        <v>0</v>
+      </c>
+      <c r="L10" t="str">
         <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
       </c>
-      <c r="L10" t="str">
+      <c r="M10" t="str">
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
-      <c r="M10" t="str">
+      <c r="N10" t="str">
         <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
       </c>
-      <c r="N10" t="str">
+      <c r="O10" t="str">
         <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
       </c>
-      <c r="O10" t="str">
-        <v/>
-      </c>
       <c r="P10" t="str">
+        <v/>
+      </c>
+      <c r="Q10" t="str">
         <v>2026-09-04T09:33:03.132Z</v>
       </c>
-      <c r="Q10" t="str">
+      <c r="R10" t="str">
         <v>2026-09-04T11:32:35.144Z</v>
       </c>
     </row>
@@ -1804,39 +2032,42 @@
         <v>Back End</v>
       </c>
       <c r="F11" t="str">
+        <v/>
+      </c>
+      <c r="G11" t="str">
         <v>2026-08-31</v>
-      </c>
-      <c r="G11" t="str">
-        <v>2026-09-04</v>
       </c>
       <c r="H11" t="str">
         <v>2026-09-04</v>
       </c>
       <c r="I11" t="str">
-        <v/>
+        <v>2026-09-04</v>
       </c>
       <c r="J11" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="K11" t="str">
+        <v>0</v>
+      </c>
+      <c r="L11" t="str">
         <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
       </c>
-      <c r="L11" t="str">
+      <c r="M11" t="str">
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
-      <c r="M11" t="str">
+      <c r="N11" t="str">
         <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
       </c>
-      <c r="N11" t="str">
+      <c r="O11" t="str">
         <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
-      <c r="O11" t="str">
-        <v/>
-      </c>
       <c r="P11" t="str">
+        <v/>
+      </c>
+      <c r="Q11" t="str">
         <v>2026-09-04T09:33:38.656Z</v>
       </c>
-      <c r="Q11" t="str">
+      <c r="R11" t="str">
         <v>2026-09-04T09:41:08.425Z</v>
       </c>
     </row>
@@ -1857,39 +2088,42 @@
         <v>Back End</v>
       </c>
       <c r="F12" t="str">
+        <v/>
+      </c>
+      <c r="G12" t="str">
         <v>2026-08-31</v>
-      </c>
-      <c r="G12" t="str">
-        <v>2026-09-04</v>
       </c>
       <c r="H12" t="str">
         <v>2026-09-04</v>
       </c>
       <c r="I12" t="str">
-        <v/>
+        <v>2026-09-04</v>
       </c>
       <c r="J12" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="K12" t="str">
+        <v>0</v>
+      </c>
+      <c r="L12" t="str">
         <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
       </c>
-      <c r="L12" t="str">
+      <c r="M12" t="str">
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
-      <c r="M12" t="str">
+      <c r="N12" t="str">
         <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
       </c>
-      <c r="N12" t="str">
+      <c r="O12" t="str">
         <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
       </c>
-      <c r="O12" t="str">
-        <v/>
-      </c>
       <c r="P12" t="str">
+        <v/>
+      </c>
+      <c r="Q12" t="str">
         <v>2026-09-04T09:34:04.072Z</v>
       </c>
-      <c r="Q12" t="str">
+      <c r="R12" t="str">
         <v>2026-09-08T07:00:11.973Z</v>
       </c>
     </row>
@@ -1910,39 +2144,42 @@
         <v>Back End</v>
       </c>
       <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13" t="str">
         <v>2026-08-24</v>
-      </c>
-      <c r="G13" t="str">
-        <v>2026-09-09</v>
       </c>
       <c r="H13" t="str">
         <v>2026-09-09</v>
       </c>
       <c r="I13" t="str">
-        <v/>
+        <v>2026-09-09</v>
       </c>
       <c r="J13" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="K13" t="str">
+        <v>0</v>
+      </c>
+      <c r="L13" t="str">
         <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
       </c>
-      <c r="L13" t="str">
+      <c r="M13" t="str">
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
-      <c r="M13" t="str">
+      <c r="N13" t="str">
         <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
       </c>
-      <c r="N13" t="str">
+      <c r="O13" t="str">
         <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
       </c>
-      <c r="O13" t="str">
-        <v/>
-      </c>
       <c r="P13" t="str">
+        <v/>
+      </c>
+      <c r="Q13" t="str">
         <v>2026-09-04T09:43:36.886Z</v>
       </c>
-      <c r="Q13" t="str">
+      <c r="R13" t="str">
         <v>2026-09-09T10:31:25.123Z</v>
       </c>
     </row>
@@ -1963,39 +2200,42 @@
         <v>Back End</v>
       </c>
       <c r="F14" t="str">
+        <v/>
+      </c>
+      <c r="G14" t="str">
         <v>2026-08-24</v>
-      </c>
-      <c r="G14" t="str">
-        <v>2026-09-09</v>
       </c>
       <c r="H14" t="str">
         <v>2026-09-09</v>
       </c>
       <c r="I14" t="str">
+        <v>2026-09-09</v>
+      </c>
+      <c r="J14" t="str">
         <v>2026-09-20</v>
       </c>
-      <c r="J14" t="str">
-        <v>0</v>
-      </c>
       <c r="K14" t="str">
+        <v>0</v>
+      </c>
+      <c r="L14" t="str">
         <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
       </c>
-      <c r="L14" t="str">
+      <c r="M14" t="str">
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
-      <c r="M14" t="str">
+      <c r="N14" t="str">
         <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
       </c>
-      <c r="N14" t="str">
+      <c r="O14" t="str">
         <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
       </c>
-      <c r="O14" t="str">
-        <v/>
-      </c>
       <c r="P14" t="str">
+        <v/>
+      </c>
+      <c r="Q14" t="str">
         <v>2026-09-04T09:43:56.520Z</v>
       </c>
-      <c r="Q14" t="str">
+      <c r="R14" t="str">
         <v>2026-09-11T06:58:59.742Z</v>
       </c>
     </row>
@@ -2016,39 +2256,42 @@
         <v>Back End</v>
       </c>
       <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15" t="str">
         <v>2026-09-07</v>
-      </c>
-      <c r="G15" t="str">
-        <v>2026-09-11</v>
       </c>
       <c r="H15" t="str">
         <v>2026-09-11</v>
       </c>
       <c r="I15" t="str">
-        <v/>
+        <v>2026-09-11</v>
       </c>
       <c r="J15" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="K15" t="str">
+        <v>0</v>
+      </c>
+      <c r="L15" t="str">
         <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
       </c>
-      <c r="L15" t="str">
+      <c r="M15" t="str">
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
-      <c r="M15" t="str">
+      <c r="N15" t="str">
         <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
       </c>
-      <c r="N15" t="str">
+      <c r="O15" t="str">
         <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
       </c>
-      <c r="O15" t="str">
-        <v/>
-      </c>
       <c r="P15" t="str">
+        <v/>
+      </c>
+      <c r="Q15" t="str">
         <v>2026-09-04T09:44:42.509Z</v>
       </c>
-      <c r="Q15" t="str">
+      <c r="R15" t="str">
         <v>2026-09-11T06:48:29.153Z</v>
       </c>
     </row>
@@ -2069,39 +2312,42 @@
         <v>Back End, Front End</v>
       </c>
       <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16" t="str">
         <v>2026-08-31</v>
-      </c>
-      <c r="G16" t="str">
-        <v>2026-09-16</v>
       </c>
       <c r="H16" t="str">
         <v>2026-09-16</v>
       </c>
       <c r="I16" t="str">
-        <v/>
+        <v>2026-09-16</v>
       </c>
       <c r="J16" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="K16" t="str">
+        <v>0</v>
+      </c>
+      <c r="L16" t="str">
         <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
       </c>
-      <c r="L16" t="str">
+      <c r="M16" t="str">
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
-      <c r="M16" t="str">
+      <c r="N16" t="str">
         <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
       </c>
-      <c r="N16" t="str">
+      <c r="O16" t="str">
         <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
       </c>
-      <c r="O16" t="str">
-        <v/>
-      </c>
       <c r="P16" t="str">
+        <v/>
+      </c>
+      <c r="Q16" t="str">
         <v>2026-09-04T09:47:39.827Z</v>
       </c>
-      <c r="Q16" t="str">
+      <c r="R16" t="str">
         <v>2026-09-04T09:47:39.843Z</v>
       </c>
     </row>
@@ -2122,39 +2368,42 @@
         <v>Back End, Front End</v>
       </c>
       <c r="F17" t="str">
+        <v/>
+      </c>
+      <c r="G17" t="str">
         <v>2026-08-31</v>
-      </c>
-      <c r="G17" t="str">
-        <v>2026-09-16</v>
       </c>
       <c r="H17" t="str">
         <v>2026-09-16</v>
       </c>
       <c r="I17" t="str">
-        <v/>
+        <v>2026-09-16</v>
       </c>
       <c r="J17" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="K17" t="str">
+        <v>0</v>
+      </c>
+      <c r="L17" t="str">
         <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
       </c>
-      <c r="L17" t="str">
+      <c r="M17" t="str">
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
-      <c r="M17" t="str">
+      <c r="N17" t="str">
         <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
       </c>
-      <c r="N17" t="str">
+      <c r="O17" t="str">
         <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
       </c>
-      <c r="O17" t="str">
-        <v/>
-      </c>
       <c r="P17" t="str">
+        <v/>
+      </c>
+      <c r="Q17" t="str">
         <v>2026-09-04T09:48:58.057Z</v>
       </c>
-      <c r="Q17" t="str">
+      <c r="R17" t="str">
         <v>2026-09-04T09:48:58.073Z</v>
       </c>
     </row>
@@ -2175,39 +2424,42 @@
         <v>Back End</v>
       </c>
       <c r="F18" t="str">
+        <v/>
+      </c>
+      <c r="G18" t="str">
         <v>2026-08-31</v>
-      </c>
-      <c r="G18" t="str">
-        <v>2026-09-18</v>
       </c>
       <c r="H18" t="str">
         <v>2026-09-18</v>
       </c>
       <c r="I18" t="str">
-        <v/>
+        <v>2026-09-18</v>
       </c>
       <c r="J18" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="K18" t="str">
+        <v>0</v>
+      </c>
+      <c r="L18" t="str">
         <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
       </c>
-      <c r="L18" t="str">
+      <c r="M18" t="str">
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
-      <c r="M18" t="str">
+      <c r="N18" t="str">
         <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
       </c>
-      <c r="N18" t="str">
+      <c r="O18" t="str">
         <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
       </c>
-      <c r="O18" t="str">
-        <v/>
-      </c>
       <c r="P18" t="str">
+        <v/>
+      </c>
+      <c r="Q18" t="str">
         <v>2026-09-04T09:50:04.917Z</v>
       </c>
-      <c r="Q18" t="str">
+      <c r="R18" t="str">
         <v>2026-09-04T10:15:31.436Z</v>
       </c>
     </row>
@@ -2228,93 +2480,100 @@
         <v>Back End</v>
       </c>
       <c r="F19" t="str">
+        <v/>
+      </c>
+      <c r="G19" t="str">
         <v>2026-08-31</v>
-      </c>
-      <c r="G19" t="str">
-        <v>2026-09-25</v>
       </c>
       <c r="H19" t="str">
         <v>2026-09-25</v>
       </c>
       <c r="I19" t="str">
-        <v/>
+        <v>2026-09-25</v>
       </c>
       <c r="J19" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="K19" t="str">
+        <v>0</v>
+      </c>
+      <c r="L19" t="str">
         <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
       </c>
-      <c r="L19" t="str">
+      <c r="M19" t="str">
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
-      <c r="M19" t="str">
+      <c r="N19" t="str">
         <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
       </c>
-      <c r="N19" t="str">
+      <c r="O19" t="str">
         <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
       </c>
-      <c r="O19" t="str">
-        <v/>
-      </c>
       <c r="P19" t="str">
+        <v/>
+      </c>
+      <c r="Q19" t="str">
         <v>2026-09-04T09:51:03.522Z</v>
       </c>
-      <c r="Q19" t="str">
+      <c r="R19" t="str">
         <v>2026-09-04T11:41:49.865Z</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" xml:space="preserve">
       <c r="A20" t="str">
         <v>576fbffe-152c-4052-834c-1d230af3784a</v>
       </c>
       <c r="B20" t="str">
         <v>แก้ไขข้อมูลนายจ้าง</v>
       </c>
-      <c r="C20" t="str">
-        <v>เพิ่มส่งสาเหตุการแก้ไขข้อมูลนายจ้าง</v>
+      <c r="C20" t="str" xml:space="preserve">
+        <v xml:space="preserve">-เพิ่มส่งสาเหตุการแก้ไขข้อมูลนายจ้าง
+-ปรับ ui ช่องค้นหาชื่อนายจาก</v>
       </c>
       <c r="D20" t="str">
         <v/>
       </c>
       <c r="E20" t="str">
-        <v>Back End</v>
+        <v>Back End, Front End</v>
       </c>
       <c r="F20" t="str">
+        <v/>
+      </c>
+      <c r="G20" t="str">
         <v>2026-09-07</v>
-      </c>
-      <c r="G20" t="str">
-        <v>2026-09-09</v>
       </c>
       <c r="H20" t="str">
         <v>2026-09-09</v>
       </c>
       <c r="I20" t="str">
+        <v>2026-09-09</v>
+      </c>
+      <c r="J20" t="str">
         <v>2026-09-13</v>
       </c>
-      <c r="J20" t="str">
-        <v>0</v>
-      </c>
       <c r="K20" t="str">
+        <v>0</v>
+      </c>
+      <c r="L20" t="str">
         <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
       </c>
-      <c r="L20" t="str">
+      <c r="M20" t="str">
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
-      <c r="M20" t="str">
+      <c r="N20" t="str">
         <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
       </c>
-      <c r="N20" t="str">
+      <c r="O20" t="str">
         <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
       </c>
-      <c r="O20" t="str">
-        <v/>
-      </c>
       <c r="P20" t="str">
+        <v/>
+      </c>
+      <c r="Q20" t="str">
         <v>2026-09-08T04:37:27.473Z</v>
       </c>
-      <c r="Q20" t="str">
-        <v>2026-09-11T06:48:10.776Z</v>
+      <c r="R20" t="str">
+        <v>2026-09-11T08:41:43.804Z</v>
       </c>
     </row>
     <row r="21">
@@ -2334,40 +2593,43 @@
         <v>Back End</v>
       </c>
       <c r="F21" t="str">
+        <v/>
+      </c>
+      <c r="G21" t="str">
         <v>2026-08-31</v>
       </c>
-      <c r="G21" t="str">
-        <v/>
-      </c>
       <c r="H21" t="str">
+        <v/>
+      </c>
+      <c r="I21" t="str">
         <v>2026-09-09</v>
       </c>
-      <c r="I21" t="str">
+      <c r="J21" t="str">
         <v>2026-09-13</v>
       </c>
-      <c r="J21" t="str">
-        <v>0</v>
-      </c>
       <c r="K21" t="str">
+        <v>0</v>
+      </c>
+      <c r="L21" t="str">
         <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
       </c>
-      <c r="L21" t="str">
+      <c r="M21" t="str">
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
-      <c r="M21" t="str">
+      <c r="N21" t="str">
         <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
       </c>
-      <c r="N21" t="str">
+      <c r="O21" t="str">
         <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
-      <c r="O21" t="str">
-        <v/>
-      </c>
       <c r="P21" t="str">
+        <v/>
+      </c>
+      <c r="Q21" t="str">
         <v>2026-09-08T07:22:24.608Z</v>
       </c>
-      <c r="Q21" t="str">
-        <v>2026-09-11T06:48:04.045Z</v>
+      <c r="R21" t="str">
+        <v>2026-09-11T08:42:08.156Z</v>
       </c>
     </row>
     <row r="22">
@@ -2384,43 +2646,46 @@
         <v/>
       </c>
       <c r="E22" t="str">
-        <v>Back End</v>
+        <v>Back End, Front End</v>
       </c>
       <c r="F22" t="str">
+        <v/>
+      </c>
+      <c r="G22" t="str">
         <v>2026-08-31</v>
       </c>
-      <c r="G22" t="str">
-        <v/>
-      </c>
       <c r="H22" t="str">
+        <v/>
+      </c>
+      <c r="I22" t="str">
         <v>2026-09-11</v>
       </c>
-      <c r="I22" t="str">
+      <c r="J22" t="str">
         <v>2026-09-13</v>
       </c>
-      <c r="J22" t="str">
-        <v>0</v>
-      </c>
       <c r="K22" t="str">
+        <v>0</v>
+      </c>
+      <c r="L22" t="str">
         <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
       </c>
-      <c r="L22" t="str">
+      <c r="M22" t="str">
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
-      <c r="M22" t="str">
+      <c r="N22" t="str">
         <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
       </c>
-      <c r="N22" t="str">
+      <c r="O22" t="str">
         <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
       </c>
-      <c r="O22" t="str">
-        <v/>
-      </c>
       <c r="P22" t="str">
+        <v/>
+      </c>
+      <c r="Q22" t="str">
         <v>2026-09-11T06:49:21.261Z</v>
       </c>
-      <c r="Q22" t="str">
-        <v>2026-09-11T06:49:25.747Z</v>
+      <c r="R22" t="str">
+        <v>2026-09-11T08:42:24.925Z</v>
       </c>
     </row>
     <row r="23" xml:space="preserve">
@@ -2441,40 +2706,43 @@
         <v>Back End</v>
       </c>
       <c r="F23" t="str">
+        <v/>
+      </c>
+      <c r="G23" t="str">
         <v>2026-09-11</v>
       </c>
-      <c r="G23" t="str">
-        <v/>
-      </c>
       <c r="H23" t="str">
+        <v/>
+      </c>
+      <c r="I23" t="str">
         <v>2026-09-14</v>
       </c>
-      <c r="I23" t="str">
+      <c r="J23" t="str">
         <v>2026-09-16</v>
       </c>
-      <c r="J23" t="str">
-        <v>0</v>
-      </c>
       <c r="K23" t="str">
+        <v>0</v>
+      </c>
+      <c r="L23" t="str">
         <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
       </c>
-      <c r="L23" t="str">
+      <c r="M23" t="str">
         <v>3663067e-457b-445c-9656-3c5886a7d364</v>
       </c>
-      <c r="M23" t="str">
+      <c r="N23" t="str">
         <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
       </c>
-      <c r="N23" t="str">
-        <v/>
-      </c>
       <c r="O23" t="str">
-        <v/>
+        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
       </c>
       <c r="P23" t="str">
+        <v/>
+      </c>
+      <c r="Q23" t="str">
         <v>2026-09-11T06:58:20.486Z</v>
       </c>
-      <c r="Q23" t="str">
-        <v>2026-09-11T06:58:20.507Z</v>
+      <c r="R23" t="str">
+        <v>2026-09-11T08:17:00.206Z</v>
       </c>
     </row>
     <row r="24">
@@ -2491,7 +2759,7 @@
         <v/>
       </c>
       <c r="E24" t="str">
-        <v>Back End</v>
+        <v>Back End, Front End</v>
       </c>
       <c r="F24" t="str">
         <v/>
@@ -2500,34 +2768,37 @@
         <v/>
       </c>
       <c r="H24" t="str">
+        <v/>
+      </c>
+      <c r="I24" t="str">
         <v>2026-08-22</v>
       </c>
-      <c r="I24" t="str">
+      <c r="J24" t="str">
         <v>2026-09-16</v>
       </c>
-      <c r="J24" t="str">
-        <v>0</v>
-      </c>
       <c r="K24" t="str">
+        <v>0</v>
+      </c>
+      <c r="L24" t="str">
         <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
       </c>
-      <c r="L24" t="str">
+      <c r="M24" t="str">
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
-      <c r="M24" t="str">
+      <c r="N24" t="str">
         <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
       </c>
-      <c r="N24" t="str">
-        <v/>
-      </c>
       <c r="O24" t="str">
-        <v/>
+        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
       </c>
       <c r="P24" t="str">
+        <v/>
+      </c>
+      <c r="Q24" t="str">
         <v>2026-09-11T06:59:51.867Z</v>
       </c>
-      <c r="Q24" t="str">
-        <v>2026-09-11T06:59:51.886Z</v>
+      <c r="R24" t="str">
+        <v>2026-09-11T08:22:00.422Z</v>
       </c>
     </row>
     <row r="25" xml:space="preserve">
@@ -2545,55 +2816,576 @@
         <v/>
       </c>
       <c r="E25" t="str">
+        <v>Back End, Front End</v>
+      </c>
+      <c r="F25" t="str">
+        <v/>
+      </c>
+      <c r="G25" t="str">
+        <v>2026-09-01</v>
+      </c>
+      <c r="H25" t="str">
+        <v/>
+      </c>
+      <c r="I25" t="str">
+        <v>2026-09-14</v>
+      </c>
+      <c r="J25" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="K25" t="str">
+        <v>0</v>
+      </c>
+      <c r="L25" t="str">
+        <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
+      </c>
+      <c r="M25" t="str">
+        <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
+      </c>
+      <c r="N25" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="O25" t="str">
+        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
+      </c>
+      <c r="P25" t="str">
+        <v/>
+      </c>
+      <c r="Q25" t="str">
+        <v>2026-09-11T07:00:25.947Z</v>
+      </c>
+      <c r="R25" t="str">
+        <v>2026-09-11T08:16:40.380Z</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>4f0a6d51-f2bc-4517-bdbe-9b39a26ebb5d</v>
+      </c>
+      <c r="B26" t="str">
+        <v>เงื่อนไขมติ 14 ก.ค.</v>
+      </c>
+      <c r="C26" t="str">
+        <v>ปรับเงื่อนไข ต่ออายุกรมธรรม์</v>
+      </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
+      <c r="E26" t="str">
         <v>Back End</v>
       </c>
-      <c r="F25" t="str">
-        <v>2026-09-01</v>
-      </c>
-      <c r="G25" t="str">
-        <v/>
-      </c>
-      <c r="H25" t="str">
-        <v>2026-09-14</v>
-      </c>
-      <c r="I25" t="str">
+      <c r="F26" t="str">
+        <v/>
+      </c>
+      <c r="G26" t="str">
+        <v/>
+      </c>
+      <c r="H26" t="str">
+        <v/>
+      </c>
+      <c r="I26" t="str">
+        <v/>
+      </c>
+      <c r="J26" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="K26" t="str">
+        <v>0</v>
+      </c>
+      <c r="L26" t="str">
+        <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
+      </c>
+      <c r="M26" t="str">
+        <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
+      </c>
+      <c r="N26" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="O26" t="str">
+        <v>55d6e756-c40c-4755-84ab-c3458437acd6</v>
+      </c>
+      <c r="P26" t="str">
+        <v/>
+      </c>
+      <c r="Q26" t="str">
+        <v>2026-09-11T07:17:53.760Z</v>
+      </c>
+      <c r="R26" t="str">
+        <v>2026-09-11T08:18:25.628Z</v>
+      </c>
+    </row>
+    <row r="27" xml:space="preserve">
+      <c r="A27" t="str">
+        <v>2033fe99-69ce-47d7-bed5-92a5d6bdedc3</v>
+      </c>
+      <c r="B27" t="str">
+        <v>เพิ่มการดักเงื่อนไขขั้นตอนลงทะเบียน</v>
+      </c>
+      <c r="C27" t="str" xml:space="preserve">
+        <v xml:space="preserve">สรุป : ดักเงื่อนไข เลขประจำตัวที่ขึ้นต้นด้วย รหัส รพ. (hcode)
+0(เลข รพ. 5 หลัก) 
+00(เลข รพ. 5 หลัก)
+000(เลข รพ. 5 หลัก) 
+เลข รพ. 5 หลัก</v>
+      </c>
+      <c r="D27" t="str" xml:space="preserve">
+        <v xml:space="preserve">massage :  “ไม่สามารถขึ้นทะเบียนได้ เนื่องจากไม่ใช่เลขแนวทางตามที่กองทุนกำหนด”
+กรณีมีเคสที่ไม่ผ่านเงื่อนไขและหลุดเข้าระบบ เป็นสถานะ ยังไม่ส่งเงิน ให้ดักเงื่อนไขห้ามออกเลขอ้างอิง และแจ้งเตือน
+massage :  “แก้ไขเลขประจำตัว เนื่องจากไม่ใช่เลขแนวทางตามที่กองทุนกำหนด”
+</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Back End</v>
+      </c>
+      <c r="F27" t="str">
+        <v/>
+      </c>
+      <c r="G27" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="H27" t="str">
+        <v/>
+      </c>
+      <c r="I27" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="J27" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="K27" t="str">
+        <v>0</v>
+      </c>
+      <c r="L27" t="str">
+        <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
+      </c>
+      <c r="M27" t="str">
+        <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
+      </c>
+      <c r="N27" t="str">
+        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+      </c>
+      <c r="O27" t="str">
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+      </c>
+      <c r="P27" t="str">
+        <v/>
+      </c>
+      <c r="Q27" t="str">
+        <v>2026-09-11T07:28:37.852Z</v>
+      </c>
+      <c r="R27" t="str">
+        <v>2026-09-11T09:14:33.049Z</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>fec6d3d9-868a-474b-b507-c36769e8db34</v>
+      </c>
+      <c r="B28" t="str">
+        <v>ส่วนลงทะเบียน</v>
+      </c>
+      <c r="C28" t="str">
+        <v xml:space="preserve"> ปรับให้ อายุ 15 ปีขึ้นไป จึงจะใส่อาชีพได้ </v>
+      </c>
+      <c r="D28" t="str">
+        <v>** ยกเว้นมติ ครม. ต้องมีอายุ 18 ขึ้นไปจึงจะใส่อาชีพได้</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Back End, Front End</v>
+      </c>
+      <c r="F28" t="str">
+        <v/>
+      </c>
+      <c r="G28" t="str">
+        <v/>
+      </c>
+      <c r="H28" t="str">
+        <v/>
+      </c>
+      <c r="I28" t="str">
+        <v/>
+      </c>
+      <c r="J28" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="K28" t="str">
+        <v>0</v>
+      </c>
+      <c r="L28" t="str">
+        <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
+      </c>
+      <c r="M28" t="str">
+        <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
+      </c>
+      <c r="N28" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="O28" t="str">
+        <v/>
+      </c>
+      <c r="P28" t="str">
+        <v/>
+      </c>
+      <c r="Q28" t="str">
+        <v>2026-09-11T07:30:13.226Z</v>
+      </c>
+      <c r="R28" t="str">
+        <v>2026-09-11T07:30:13.237Z</v>
+      </c>
+    </row>
+    <row r="29" xml:space="preserve">
+      <c r="A29" t="str">
+        <v>2702b682-23d0-4b69-a895-7bd6d6a3965f</v>
+      </c>
+      <c r="B29" t="str">
+        <v>เรียงลำดับเมนูใหม่</v>
+      </c>
+      <c r="C29" t="str" xml:space="preserve">
+        <v xml:space="preserve">1.การขึ้นทะเบียน
+2.ผู้มีสิทธิประกันสุขภาพ
+3.การจ่ายชดเชย
+4.Dashboard พื้นที่นำร่อง
+ </v>
+      </c>
+      <c r="D29" t="str">
+        <v/>
+      </c>
+      <c r="E29" t="str">
+        <v>Front End</v>
+      </c>
+      <c r="F29" t="str">
+        <v/>
+      </c>
+      <c r="G29" t="str">
+        <v/>
+      </c>
+      <c r="H29" t="str">
+        <v/>
+      </c>
+      <c r="I29" t="str">
         <v>2026-09-16</v>
       </c>
-      <c r="J25" t="str">
-        <v>0</v>
-      </c>
-      <c r="K25" t="str">
+      <c r="J29" t="str">
+        <v/>
+      </c>
+      <c r="K29" t="str">
+        <v>0</v>
+      </c>
+      <c r="L29" t="str">
         <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
       </c>
-      <c r="L25" t="str">
+      <c r="M29" t="str">
+        <v>4480c937-7ac8-4ba9-a170-9071fbd4749a</v>
+      </c>
+      <c r="N29" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="O29" t="str">
+        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
+      </c>
+      <c r="P29" t="str">
+        <v/>
+      </c>
+      <c r="Q29" t="str">
+        <v>2026-09-11T07:31:09.231Z</v>
+      </c>
+      <c r="R29" t="str">
+        <v>2026-09-11T08:22:33.274Z</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>a3bbee49-623f-4bc2-935b-a989adca81ca</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Dashboard</v>
+      </c>
+      <c r="C30" t="str">
+        <v>เพิ่ม % สถานะการชำระเงินค่าประกันสุขภาพ</v>
+      </c>
+      <c r="D30" t="str">
+        <v/>
+      </c>
+      <c r="E30" t="str">
+        <v>Back End, Front End</v>
+      </c>
+      <c r="F30" t="str">
+        <v/>
+      </c>
+      <c r="G30" t="str">
+        <v/>
+      </c>
+      <c r="H30" t="str">
+        <v/>
+      </c>
+      <c r="I30" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="J30" t="str">
+        <v/>
+      </c>
+      <c r="K30" t="str">
+        <v>0</v>
+      </c>
+      <c r="L30" t="str">
+        <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
+      </c>
+      <c r="M30" t="str">
+        <v>4480c937-7ac8-4ba9-a170-9071fbd4749a</v>
+      </c>
+      <c r="N30" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="O30" t="str">
+        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
+      </c>
+      <c r="P30" t="str">
+        <v/>
+      </c>
+      <c r="Q30" t="str">
+        <v>2026-09-11T07:31:32.339Z</v>
+      </c>
+      <c r="R30" t="str">
+        <v>2026-09-11T08:22:44.204Z</v>
+      </c>
+    </row>
+    <row r="31" xml:space="preserve">
+      <c r="A31" t="str">
+        <v>46019afc-2896-43ad-821c-552404768662</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Dashboard หน่วยบริการที่มีผู้มัสิทธิประกันสุขภาพทั้งหมด 10 อันดับ</v>
+      </c>
+      <c r="C31" t="str" xml:space="preserve">
+        <v xml:space="preserve">กรณี สสจ. ให้แสดง รพ. ทั้งหมดใน สสจ.
+กรณี รพ. ให้แสดงเฉพาะของ รพ. ตนเอง
+กรณี แอดมิน ให้แสดง รพ. ทั้งหมด</v>
+      </c>
+      <c r="D31" t="str">
+        <v/>
+      </c>
+      <c r="E31" t="str">
+        <v>Back End</v>
+      </c>
+      <c r="F31" t="str">
+        <v/>
+      </c>
+      <c r="G31" t="str">
+        <v/>
+      </c>
+      <c r="H31" t="str">
+        <v/>
+      </c>
+      <c r="I31" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="J31" t="str">
+        <v/>
+      </c>
+      <c r="K31" t="str">
+        <v>0</v>
+      </c>
+      <c r="L31" t="str">
+        <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
+      </c>
+      <c r="M31" t="str">
+        <v>4480c937-7ac8-4ba9-a170-9071fbd4749a</v>
+      </c>
+      <c r="N31" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="O31" t="str">
+        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
+      </c>
+      <c r="P31" t="str">
+        <v/>
+      </c>
+      <c r="Q31" t="str">
+        <v>2026-09-11T07:32:44.530Z</v>
+      </c>
+      <c r="R31" t="str">
+        <v>2026-09-11T08:34:52.111Z</v>
+      </c>
+    </row>
+    <row r="32" xml:space="preserve">
+      <c r="A32" t="str">
+        <v>c0a292e6-7ae6-4e30-a09f-b6551efd53a4</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Dashboard  โรคที่มีการจ่ายชดเชยค่าบริการทางการแพทย์สูงสุด 10 อันดับ  IPD,OPD</v>
+      </c>
+      <c r="C32" t="str" xml:space="preserve">
+        <v xml:space="preserve">สรุป :  ให้แสดงเฉพาะรายการที่มีข้อมูล
+</v>
+      </c>
+      <c r="D32" t="str">
+        <v/>
+      </c>
+      <c r="E32" t="str">
+        <v>Back End, Front End</v>
+      </c>
+      <c r="F32" t="str">
+        <v/>
+      </c>
+      <c r="G32" t="str">
+        <v/>
+      </c>
+      <c r="H32" t="str">
+        <v/>
+      </c>
+      <c r="I32" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="J32" t="str">
+        <v/>
+      </c>
+      <c r="K32" t="str">
+        <v>0</v>
+      </c>
+      <c r="L32" t="str">
+        <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
+      </c>
+      <c r="M32" t="str">
+        <v>4480c937-7ac8-4ba9-a170-9071fbd4749a</v>
+      </c>
+      <c r="N32" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="O32" t="str">
+        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
+      </c>
+      <c r="P32" t="str">
+        <v/>
+      </c>
+      <c r="Q32" t="str">
+        <v>2026-09-11T07:33:50.111Z</v>
+      </c>
+      <c r="R32" t="str">
+        <v>2026-09-11T08:23:10.535Z</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>ada990db-b47a-4ec0-b8c6-03c068f69af6</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Log</v>
+      </c>
+      <c r="C33" t="str">
+        <v>ให้แสดงข้อมูลของ รพ. ตามรายชื่อ ที่กองทุนส่งให้</v>
+      </c>
+      <c r="D33" t="str">
+        <v/>
+      </c>
+      <c r="E33" t="str">
+        <v>Back End, Front End</v>
+      </c>
+      <c r="F33" t="str">
+        <v/>
+      </c>
+      <c r="G33" t="str">
+        <v/>
+      </c>
+      <c r="H33" t="str">
+        <v/>
+      </c>
+      <c r="I33" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="J33" t="str">
+        <v/>
+      </c>
+      <c r="K33" t="str">
+        <v>0</v>
+      </c>
+      <c r="L33" t="str">
+        <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
+      </c>
+      <c r="M33" t="str">
+        <v>4480c937-7ac8-4ba9-a170-9071fbd4749a</v>
+      </c>
+      <c r="N33" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="O33" t="str">
+        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
+      </c>
+      <c r="P33" t="str">
+        <v/>
+      </c>
+      <c r="Q33" t="str">
+        <v>2026-09-11T07:34:25.172Z</v>
+      </c>
+      <c r="R33" t="str">
+        <v>2026-09-11T08:23:27.693Z</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>4aef4aa0-8e8b-4280-b75a-f6df9d48e73a</v>
+      </c>
+      <c r="B34" t="str">
+        <v>ตรวจสอบ และดักเงื่อนไขเลขที่สามารถลงทะเบียนได้</v>
+      </c>
+      <c r="C34" t="str">
+        <v>จากเอกสารที่สามารถซื้อประกันสุขภาพได้</v>
+      </c>
+      <c r="D34" t="str">
+        <v>FE เอาดักจำนวน passprot_no ออกแต่ตั้งขึ้นต้นด้วย ภาษาอังกฤษ ตามด้วยเลข</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Back End, Front End</v>
+      </c>
+      <c r="F34" t="str">
+        <v/>
+      </c>
+      <c r="G34" t="str">
+        <v/>
+      </c>
+      <c r="H34" t="str">
+        <v/>
+      </c>
+      <c r="I34" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="J34" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="K34" t="str">
+        <v>0</v>
+      </c>
+      <c r="L34" t="str">
+        <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
+      </c>
+      <c r="M34" t="str">
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
-      <c r="M25" t="str">
-        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
-      </c>
-      <c r="N25" t="str">
-        <v/>
-      </c>
-      <c r="O25" t="str">
-        <v/>
-      </c>
-      <c r="P25" t="str">
-        <v>2026-09-11T07:00:25.947Z</v>
-      </c>
-      <c r="Q25" t="str">
-        <v>2026-09-11T07:00:25.966Z</v>
+      <c r="N34" t="str">
+        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+      </c>
+      <c r="O34" t="str">
+        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
+      </c>
+      <c r="P34" t="str">
+        <v/>
+      </c>
+      <c r="Q34" t="str">
+        <v>2026-09-11T07:35:13.899Z</v>
+      </c>
+      <c r="R34" t="str">
+        <v>2026-09-11T09:14:25.182Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R34"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I59"/>
+  <dimension ref="A1:I71"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4306,16 +5098,364 @@
         <v>2026-09-11T07:00:25.995Z</v>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>0057271c-ddfc-4aa9-a9c7-e889d0d7550a</v>
+      </c>
+      <c r="B60" t="str">
+        <v>4f0a6d51-f2bc-4517-bdbe-9b39a26ebb5d</v>
+      </c>
+      <c r="C60" t="str">
+        <v/>
+      </c>
+      <c r="D60" t="str">
+        <v/>
+      </c>
+      <c r="E60" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="F60" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="G60" t="str">
+        <v>2026-09-11T07:17:53.786Z</v>
+      </c>
+      <c r="H60" t="str">
+        <v>2026-09-11T07:17:53.789Z</v>
+      </c>
+      <c r="I60" t="str">
+        <v>2026-09-11T07:17:53.789Z</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>f9d1655c-9ebc-4f9b-a92b-805f78758f0e</v>
+      </c>
+      <c r="B61" t="str">
+        <v>2033fe99-69ce-47d7-bed5-92a5d6bdedc3</v>
+      </c>
+      <c r="C61" t="str">
+        <v/>
+      </c>
+      <c r="D61" t="str">
+        <v/>
+      </c>
+      <c r="E61" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="F61" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="G61" t="str">
+        <v>2026-09-11T07:28:37.909Z</v>
+      </c>
+      <c r="H61" t="str">
+        <v>2026-09-11T07:28:37.911Z</v>
+      </c>
+      <c r="I61" t="str">
+        <v>2026-09-11T07:28:37.911Z</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>ede20937-8ef6-4570-a63b-99a111128087</v>
+      </c>
+      <c r="B62" t="str">
+        <v>fec6d3d9-868a-474b-b507-c36769e8db34</v>
+      </c>
+      <c r="C62" t="str">
+        <v/>
+      </c>
+      <c r="D62" t="str">
+        <v/>
+      </c>
+      <c r="E62" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="F62" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="G62" t="str">
+        <v>2026-09-11T07:30:13.251Z</v>
+      </c>
+      <c r="H62" t="str">
+        <v>2026-09-11T07:30:13.253Z</v>
+      </c>
+      <c r="I62" t="str">
+        <v>2026-09-11T07:30:13.253Z</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>6d4d1e07-cd63-4281-a2f3-da7f352e1c78</v>
+      </c>
+      <c r="B63" t="str">
+        <v>2702b682-23d0-4b69-a895-7bd6d6a3965f</v>
+      </c>
+      <c r="C63" t="str">
+        <v/>
+      </c>
+      <c r="D63" t="str">
+        <v/>
+      </c>
+      <c r="E63" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="F63" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="G63" t="str">
+        <v>2026-09-11T07:31:09.256Z</v>
+      </c>
+      <c r="H63" t="str">
+        <v>2026-09-11T07:31:09.258Z</v>
+      </c>
+      <c r="I63" t="str">
+        <v>2026-09-11T07:31:09.258Z</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>f9361654-42be-48e4-9071-7c8faf2b29f9</v>
+      </c>
+      <c r="B64" t="str">
+        <v>a3bbee49-623f-4bc2-935b-a989adca81ca</v>
+      </c>
+      <c r="C64" t="str">
+        <v/>
+      </c>
+      <c r="D64" t="str">
+        <v/>
+      </c>
+      <c r="E64" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="F64" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="G64" t="str">
+        <v>2026-09-11T07:31:32.364Z</v>
+      </c>
+      <c r="H64" t="str">
+        <v>2026-09-11T07:31:32.366Z</v>
+      </c>
+      <c r="I64" t="str">
+        <v>2026-09-11T07:31:32.366Z</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>fd3d3501-5b18-40a8-acad-2e3eaeaa4a9a</v>
+      </c>
+      <c r="B65" t="str">
+        <v>46019afc-2896-43ad-821c-552404768662</v>
+      </c>
+      <c r="C65" t="str">
+        <v/>
+      </c>
+      <c r="D65" t="str">
+        <v/>
+      </c>
+      <c r="E65" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="F65" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="G65" t="str">
+        <v>2026-09-11T07:32:44.557Z</v>
+      </c>
+      <c r="H65" t="str">
+        <v>2026-09-11T07:32:44.559Z</v>
+      </c>
+      <c r="I65" t="str">
+        <v>2026-09-11T07:32:44.559Z</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>5b89bcf2-84e2-4b3d-bebd-1725fe0f3233</v>
+      </c>
+      <c r="B66" t="str">
+        <v>c0a292e6-7ae6-4e30-a09f-b6551efd53a4</v>
+      </c>
+      <c r="C66" t="str">
+        <v/>
+      </c>
+      <c r="D66" t="str">
+        <v/>
+      </c>
+      <c r="E66" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="F66" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="G66" t="str">
+        <v>2026-09-11T07:33:50.138Z</v>
+      </c>
+      <c r="H66" t="str">
+        <v>2026-09-11T07:33:50.140Z</v>
+      </c>
+      <c r="I66" t="str">
+        <v>2026-09-11T07:33:50.140Z</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>3c49dc6c-9d35-49cf-9d9b-90266b33a15f</v>
+      </c>
+      <c r="B67" t="str">
+        <v>ada990db-b47a-4ec0-b8c6-03c068f69af6</v>
+      </c>
+      <c r="C67" t="str">
+        <v/>
+      </c>
+      <c r="D67" t="str">
+        <v/>
+      </c>
+      <c r="E67" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="F67" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="G67" t="str">
+        <v>2026-09-11T07:34:25.200Z</v>
+      </c>
+      <c r="H67" t="str">
+        <v>2026-09-11T07:34:25.202Z</v>
+      </c>
+      <c r="I67" t="str">
+        <v>2026-09-11T07:34:25.202Z</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>840ee878-7ccf-4bdf-bb7d-0bfc1bb4cb0c</v>
+      </c>
+      <c r="B68" t="str">
+        <v>4aef4aa0-8e8b-4280-b75a-f6df9d48e73a</v>
+      </c>
+      <c r="C68" t="str">
+        <v/>
+      </c>
+      <c r="D68" t="str">
+        <v/>
+      </c>
+      <c r="E68" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="F68" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="G68" t="str">
+        <v>2026-09-11T07:35:13.927Z</v>
+      </c>
+      <c r="H68" t="str">
+        <v>2026-09-11T07:35:13.929Z</v>
+      </c>
+      <c r="I68" t="str">
+        <v>2026-09-11T07:35:13.929Z</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>d596d1f3-8b68-4681-9fc2-1bf4739246ce</v>
+      </c>
+      <c r="B69" t="str">
+        <v>4aef4aa0-8e8b-4280-b75a-f6df9d48e73a</v>
+      </c>
+      <c r="C69" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="D69" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="E69" t="str">
+        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+      </c>
+      <c r="F69" t="str">
+        <v>In Progress</v>
+      </c>
+      <c r="G69" t="str">
+        <v>2026-09-11T08:53:06.352Z</v>
+      </c>
+      <c r="H69" t="str">
+        <v>2026-09-11T08:53:06.357Z</v>
+      </c>
+      <c r="I69" t="str">
+        <v>2026-09-11T08:53:06.357Z</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>be540310-3ba5-44bb-a3f8-eb4d76d6b47f</v>
+      </c>
+      <c r="B70" t="str">
+        <v>2033fe99-69ce-47d7-bed5-92a5d6bdedc3</v>
+      </c>
+      <c r="C70" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="D70" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="E70" t="str">
+        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+      </c>
+      <c r="F70" t="str">
+        <v>In Progress</v>
+      </c>
+      <c r="G70" t="str">
+        <v>2026-09-11T08:53:10.245Z</v>
+      </c>
+      <c r="H70" t="str">
+        <v>2026-09-11T08:53:10.248Z</v>
+      </c>
+      <c r="I70" t="str">
+        <v>2026-09-11T08:53:10.248Z</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>bc187da1-5dbf-4a9f-a160-2d7b3592a1bd</v>
+      </c>
+      <c r="B71" t="str">
+        <v>e323d9c8-295f-472c-93f3-fefc39655d80</v>
+      </c>
+      <c r="C71" t="str">
+        <v>f568698e-99c5-418d-8036-5f99072d6e28</v>
+      </c>
+      <c r="D71" t="str">
+        <v>Modify</v>
+      </c>
+      <c r="E71" t="str">
+        <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
+      </c>
+      <c r="F71" t="str">
+        <v>UAT</v>
+      </c>
+      <c r="G71" t="str">
+        <v>2026-09-11T09:28:49.708Z</v>
+      </c>
+      <c r="H71" t="str">
+        <v>2026-09-11T09:28:49.712Z</v>
+      </c>
+      <c r="I71" t="str">
+        <v>2026-09-11T09:28:49.712Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I59"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I71"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4342,267 +5482,359 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>e5435e0d-9a20-4241-adc6-e880dc6bd3d2</v>
+        <v>c9699cc1-1683-4feb-984e-878d32682885</v>
       </c>
       <c r="B2" t="str">
         <v>e323d9c8-295f-472c-93f3-fefc39655d80</v>
       </c>
       <c r="C2" t="str">
-        <v>ผลตรวจสุขภาพ สัมพันธ์กับสรุปผลการตรวจสุขภาพ</v>
+        <v>ผลการตรวจการตั้งครรภ์ ถ้าติ๊ก ตั้งครรภ์ ช่องผลการตรวจวัณโรคกับผลการตรวจโรคเท้าช้าง ให้เป็นทึบไปเลย เพราะไม่ได้มีการตรวจ</v>
       </c>
       <c r="D2" t="str">
         <v>TRUE</v>
       </c>
       <c r="E2" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-09-04T09:28:44.731Z</v>
+        <v>2026-09-04T09:28:53.342Z</v>
       </c>
       <c r="G2" t="str">
-        <v>2026-09-04T10:15:49.842Z</v>
+        <v>2026-09-04T10:15:50.555Z</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>c9699cc1-1683-4feb-984e-878d32682885</v>
+        <v>4657d602-61e3-4999-8fd6-2b2eda534e20</v>
       </c>
       <c r="B3" t="str">
         <v>e323d9c8-295f-472c-93f3-fefc39655d80</v>
       </c>
       <c r="C3" t="str">
-        <v>ผลการตรวจการตั้งครรภ์ ถ้าติ๊ก ตั้งครรภ์ ช่องผลการตรวจวัณโรคกับผลการตรวจโรคเท้าช้าง ให้เป็นทึบไปเลย เพราะไม่ได้มีการตรวจ</v>
+        <v>ส่วนใบรับรองแพทย์ ถ้า ผ่าน = สีเขียว, ประเภท 2 = สีเหลือง, ประเภท 3 = สีแดง</v>
       </c>
       <c r="D3" t="str">
         <v>TRUE</v>
       </c>
       <c r="E3" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F3" t="str">
-        <v>2026-09-04T09:28:53.342Z</v>
+        <v>2026-09-04T09:29:00.544Z</v>
       </c>
       <c r="G3" t="str">
-        <v>2026-09-04T10:15:50.555Z</v>
+        <v>2026-09-11T08:28:50.401Z</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>4657d602-61e3-4999-8fd6-2b2eda534e20</v>
+        <v>47e9f838-dea2-451c-a4a6-7ad29c961c4a</v>
       </c>
       <c r="B4" t="str">
-        <v>e323d9c8-295f-472c-93f3-fefc39655d80</v>
+        <v>e49e5c13-9c33-449b-9c2c-3b48f3119d16</v>
       </c>
       <c r="C4" t="str">
-        <v>ส่วนใบรับรองแพทย์ ถ้า ผ่าน = สีเขียว, ประเภท 2 = สีเหลือง, ประเภท 3 = สีแดง</v>
+        <v>Log ใบรับรองแพทย์ Collection ใหม่</v>
       </c>
       <c r="D4" t="str">
-        <v>TRUE</v>
+        <v>FALSE</v>
       </c>
       <c r="E4" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F4" t="str">
-        <v>2026-09-04T09:29:00.544Z</v>
+        <v>2026-09-04T09:50:19.826Z</v>
       </c>
       <c r="G4" t="str">
-        <v>2026-09-04T10:15:51.145Z</v>
+        <v>2026-09-04T10:15:29.325Z</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>47e9f838-dea2-451c-a4a6-7ad29c961c4a</v>
+        <v>e7249296-600f-447c-9869-1d67655b3075</v>
       </c>
       <c r="B5" t="str">
         <v>e49e5c13-9c33-449b-9c2c-3b48f3119d16</v>
       </c>
       <c r="C5" t="str">
-        <v>Log ใบรับรองแพทย์ Collection ใหม่</v>
+        <v>Log กรมธรรม์ไปใช้ Collection ใหม่</v>
       </c>
       <c r="D5" t="str">
         <v>FALSE</v>
       </c>
       <c r="E5" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F5" t="str">
-        <v>2026-09-04T09:50:19.826Z</v>
+        <v>2026-09-04T09:50:30.949Z</v>
       </c>
       <c r="G5" t="str">
-        <v>2026-09-04T10:15:29.325Z</v>
+        <v>2026-09-04T10:15:28.638Z</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>e7249296-600f-447c-9869-1d67655b3075</v>
+        <v>b8311bf6-ddb0-4b10-9dae-f25584050fae</v>
       </c>
       <c r="B6" t="str">
-        <v>e49e5c13-9c33-449b-9c2c-3b48f3119d16</v>
+        <v>81722c13-7a3f-4789-a1ac-a70c472369e0</v>
       </c>
       <c r="C6" t="str">
-        <v>Log กรมธรรม์ไปใช้ Collection ใหม่</v>
+        <v>เพิ่ม Log จัดการสิทธิ และแสดงข้อมูล</v>
       </c>
       <c r="D6" t="str">
         <v>FALSE</v>
       </c>
       <c r="E6" t="str">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F6" t="str">
-        <v>2026-09-04T09:50:30.949Z</v>
+        <v>2026-09-04T09:51:24.363Z</v>
       </c>
       <c r="G6" t="str">
-        <v>2026-09-04T10:15:28.638Z</v>
+        <v>2026-09-04T10:15:37.156Z</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>b8311bf6-ddb0-4b10-9dae-f25584050fae</v>
+        <v>168a98f3-0cdb-4081-8b06-92fc6a1b4f97</v>
       </c>
       <c r="B7" t="str">
         <v>81722c13-7a3f-4789-a1ac-a70c472369e0</v>
       </c>
       <c r="C7" t="str">
-        <v>เพิ่ม Log จัดการสิทธิ และแสดงข้อมูล</v>
+        <v>เพิ่ม Log ลายเซ็น และแสดงข้อมูล</v>
       </c>
       <c r="D7" t="str">
         <v>FALSE</v>
       </c>
       <c r="E7" t="str">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F7" t="str">
-        <v>2026-09-04T09:51:24.363Z</v>
+        <v>2026-09-04T09:51:30.264Z</v>
       </c>
       <c r="G7" t="str">
-        <v>2026-09-04T10:15:37.156Z</v>
+        <v>2026-09-04T10:15:37.653Z</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>168a98f3-0cdb-4081-8b06-92fc6a1b4f97</v>
+        <v>78826565-b6f0-4134-8ec5-51b689568502</v>
       </c>
       <c r="B8" t="str">
         <v>81722c13-7a3f-4789-a1ac-a70c472369e0</v>
       </c>
       <c r="C8" t="str">
-        <v>เพิ่ม Log ลายเซ็น และแสดงข้อมูล</v>
+        <v>เพิ่ม Log ตั้งค่าระบบ และแสดงข้อมูล</v>
       </c>
       <c r="D8" t="str">
         <v>FALSE</v>
       </c>
       <c r="E8" t="str">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F8" t="str">
-        <v>2026-09-04T09:51:30.264Z</v>
+        <v>2026-09-04T09:51:37.463Z</v>
       </c>
       <c r="G8" t="str">
-        <v>2026-09-04T10:15:37.653Z</v>
+        <v>2026-09-04T10:15:38.297Z</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>78826565-b6f0-4134-8ec5-51b689568502</v>
+        <v>d3abd120-8ba6-4dca-b36e-64c8291bcc93</v>
       </c>
       <c r="B9" t="str">
         <v>81722c13-7a3f-4789-a1ac-a70c472369e0</v>
       </c>
       <c r="C9" t="str">
-        <v>เพิ่ม Log ตั้งค่าระบบ และแสดงข้อมูล</v>
+        <v>ปรับ Log Statement Collection ใหม่</v>
       </c>
       <c r="D9" t="str">
         <v>FALSE</v>
       </c>
       <c r="E9" t="str">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F9" t="str">
-        <v>2026-09-04T09:51:37.463Z</v>
+        <v>2026-09-04T09:51:43.481Z</v>
       </c>
       <c r="G9" t="str">
-        <v>2026-09-04T10:15:38.297Z</v>
+        <v>2026-09-04T11:41:47.445Z</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>d3abd120-8ba6-4dca-b36e-64c8291bcc93</v>
+        <v>ba295d36-7862-4119-9b75-ab172c89a88e</v>
       </c>
       <c r="B10" t="str">
-        <v>81722c13-7a3f-4789-a1ac-a70c472369e0</v>
+        <v>e323d9c8-295f-472c-93f3-fefc39655d80</v>
       </c>
       <c r="C10" t="str">
-        <v>ปรับ Log Statement Collection ใหม่</v>
+        <v>แก้ไขเงื่อนไขสรุปผลตรวจสุขภาพ</v>
       </c>
       <c r="D10" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
       </c>
       <c r="E10" t="str">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F10" t="str">
-        <v>2026-09-04T09:51:43.481Z</v>
+        <v>2026-09-11T06:56:01.870Z</v>
       </c>
       <c r="G10" t="str">
-        <v>2026-09-04T11:41:47.445Z</v>
+        <v>2026-09-11T08:28:49.110Z</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>30680aff-dffc-4170-9152-67ee539b3e93</v>
+        <v>bfe255cd-98bd-40a3-96e1-ab996fe7202c</v>
       </c>
       <c r="B11" t="str">
-        <v>e323d9c8-295f-472c-93f3-fefc39655d80</v>
+        <v>2033fe99-69ce-47d7-bed5-92a5d6bdedc3</v>
       </c>
       <c r="C11" t="str">
-        <v>ปรับสีสถานะเพิ่มความเข็มขึ้น</v>
+        <v>ลงทะเบียน Draf</v>
       </c>
       <c r="D11" t="str">
         <v>FALSE</v>
       </c>
       <c r="E11" t="str">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F11" t="str">
-        <v>2026-09-11T06:55:08.648Z</v>
+        <v>2026-09-11T07:28:37.879Z</v>
       </c>
       <c r="G11" t="str">
-        <v>2026-09-11T06:55:12.799Z</v>
+        <v>2026-09-11T08:17:31.114Z</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>ba295d36-7862-4119-9b75-ab172c89a88e</v>
+        <v>f17a5ff5-5c29-4c90-a446-189127086d64</v>
       </c>
       <c r="B12" t="str">
-        <v>e323d9c8-295f-472c-93f3-fefc39655d80</v>
+        <v>2033fe99-69ce-47d7-bed5-92a5d6bdedc3</v>
       </c>
       <c r="C12" t="str">
-        <v>แก้ไขเงื่อนไขสรุปผลตรวจสุขภาพ</v>
+        <v>ลงทะเบียนออก FCODE</v>
       </c>
       <c r="D12" t="str">
         <v>FALSE</v>
       </c>
       <c r="E12" t="str">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F12" t="str">
-        <v>2026-09-11T06:56:01.870Z</v>
+        <v>2026-09-11T07:28:37.884Z</v>
       </c>
       <c r="G12" t="str">
-        <v>2026-09-11T06:56:01.870Z</v>
+        <v>2026-09-11T08:17:32.845Z</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>4edb6864-2622-4350-b92b-c0c48bbb8deb</v>
+      </c>
+      <c r="B13" t="str">
+        <v>2033fe99-69ce-47d7-bed5-92a5d6bdedc3</v>
+      </c>
+      <c r="C13" t="str">
+        <v>แก้ไขข้อมูล Draf</v>
+      </c>
+      <c r="D13" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="E13" t="str">
+        <v>2</v>
+      </c>
+      <c r="F13" t="str">
+        <v>2026-09-11T07:28:37.890Z</v>
+      </c>
+      <c r="G13" t="str">
+        <v>2026-09-11T08:17:33.478Z</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>65a8c469-13cb-4029-84bb-d97fbfe839b5</v>
+      </c>
+      <c r="B14" t="str">
+        <v>2033fe99-69ce-47d7-bed5-92a5d6bdedc3</v>
+      </c>
+      <c r="C14" t="str">
+        <v>แก้ไขข้อมูล</v>
+      </c>
+      <c r="D14" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="E14" t="str">
+        <v>3</v>
+      </c>
+      <c r="F14" t="str">
+        <v>2026-09-11T07:28:37.896Z</v>
+      </c>
+      <c r="G14" t="str">
+        <v>2026-09-11T08:17:34.246Z</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>425ff6e2-40e5-41fd-bb1a-ef0a523ee4c5</v>
+      </c>
+      <c r="B15" t="str">
+        <v>2033fe99-69ce-47d7-bed5-92a5d6bdedc3</v>
+      </c>
+      <c r="C15" t="str">
+        <v>ออกเลขอ้างอิง</v>
+      </c>
+      <c r="D15" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="E15" t="str">
+        <v>4</v>
+      </c>
+      <c r="F15" t="str">
+        <v>2026-09-11T07:28:37.901Z</v>
+      </c>
+      <c r="G15" t="str">
+        <v>2026-09-11T08:17:34.792Z</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>c577077b-27fa-405a-b8f9-50fb7f3f2550</v>
+      </c>
+      <c r="B16" t="str">
+        <v>2033fe99-69ce-47d7-bed5-92a5d6bdedc3</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Import ข้อมูลลงทะเบียน</v>
+      </c>
+      <c r="D16" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="E16" t="str">
+        <v>11</v>
+      </c>
+      <c r="F16" t="str">
+        <v>2026-09-11T07:35:45.698Z</v>
+      </c>
+      <c r="G16" t="str">
+        <v>2026-09-11T08:17:36.029Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G16"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F54"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5166,10 +6398,10 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>20bd867f-f75b-4d0b-8041-ab6406c30788</v>
+        <v>260bb430-4d1d-4d94-933e-83126ec77f7c</v>
       </c>
       <c r="B29" t="str">
-        <v>c1b2bc1d-f4c5-42ea-bdc8-4fdc41bfd8ee</v>
+        <v>1e95dc95-6f63-4810-9d57-8520eb9b42c5</v>
       </c>
       <c r="C29" t="str">
         <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
@@ -5178,155 +6410,515 @@
         <v>0</v>
       </c>
       <c r="E29" t="str">
-        <v>2026-09-11T06:48:04.034Z</v>
+        <v>2026-09-11T06:49:45.495Z</v>
       </c>
       <c r="F29" t="str">
-        <v>2026-09-11T06:48:04.034Z</v>
+        <v>2026-09-11T06:49:45.495Z</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>9858a349-bd2a-4b33-99a3-dcd1a4e0023c</v>
+        <v>96cc8b37-e673-419a-bf8d-08393ece27ae</v>
       </c>
       <c r="B30" t="str">
-        <v>576fbffe-152c-4052-834c-1d230af3784a</v>
+        <v>6ac09b86-b7ee-4b62-b048-4594eca71b6c</v>
       </c>
       <c r="C30" t="str">
-        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
+        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
       </c>
       <c r="D30" t="str">
         <v>0</v>
       </c>
       <c r="E30" t="str">
-        <v>2026-09-11T06:48:10.741Z</v>
+        <v>2026-09-11T06:58:59.731Z</v>
       </c>
       <c r="F30" t="str">
-        <v>2026-09-11T06:48:10.741Z</v>
+        <v>2026-09-11T06:58:59.731Z</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>a491ec90-2d22-49e2-832d-a5c7e77f3802</v>
+        <v>475f6552-8f0d-4341-bafb-d3ef407ca908</v>
       </c>
       <c r="B31" t="str">
-        <v>576fbffe-152c-4052-834c-1d230af3784a</v>
+        <v>db57a402-f79a-4e85-9c0f-e0aa07395e56</v>
       </c>
       <c r="C31" t="str">
-        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
       </c>
       <c r="D31" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E31" t="str">
-        <v>2026-09-11T06:48:10.757Z</v>
+        <v>2026-09-11T08:16:40.364Z</v>
       </c>
       <c r="F31" t="str">
-        <v>2026-09-11T06:48:10.757Z</v>
+        <v>2026-09-11T08:16:40.364Z</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>de6dc226-235c-4da0-a30f-e75d4aca61e5</v>
+        <v>80792acf-bd23-453f-bf35-a88a789081f9</v>
       </c>
       <c r="B32" t="str">
-        <v>a2d08247-d1c8-4c29-9663-96adb51418ff</v>
+        <v>db57a402-f79a-4e85-9c0f-e0aa07395e56</v>
       </c>
       <c r="C32" t="str">
-        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
+        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
       </c>
       <c r="D32" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E32" t="str">
-        <v>2026-09-11T06:49:21.285Z</v>
+        <v>2026-09-11T08:16:40.372Z</v>
       </c>
       <c r="F32" t="str">
-        <v>2026-09-11T06:49:21.285Z</v>
+        <v>2026-09-11T08:16:40.372Z</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>d99f05b1-5193-452c-b1ac-afbc759d8cac</v>
+        <v>234de469-7c7e-46b7-97c9-a8643e71a848</v>
       </c>
       <c r="B33" t="str">
-        <v>a2d08247-d1c8-4c29-9663-96adb51418ff</v>
+        <v>61dd30f5-4dcd-42a8-a3f7-19c95b56a2fc</v>
       </c>
       <c r="C33" t="str">
-        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
       </c>
       <c r="D33" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E33" t="str">
-        <v>2026-09-11T06:49:21.297Z</v>
+        <v>2026-09-11T08:17:00.186Z</v>
       </c>
       <c r="F33" t="str">
-        <v>2026-09-11T06:49:21.297Z</v>
+        <v>2026-09-11T08:17:00.186Z</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>260bb430-4d1d-4d94-933e-83126ec77f7c</v>
+        <v>53821444-cde2-4a76-a6f3-d8fc9bafe86e</v>
       </c>
       <c r="B34" t="str">
-        <v>1e95dc95-6f63-4810-9d57-8520eb9b42c5</v>
+        <v>61dd30f5-4dcd-42a8-a3f7-19c95b56a2fc</v>
       </c>
       <c r="C34" t="str">
-        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
       </c>
       <c r="D34" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E34" t="str">
-        <v>2026-09-11T06:49:45.495Z</v>
+        <v>2026-09-11T08:17:00.198Z</v>
       </c>
       <c r="F34" t="str">
-        <v>2026-09-11T06:49:45.495Z</v>
+        <v>2026-09-11T08:17:00.198Z</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>5f14d6ba-83fa-45f2-b869-5981498a8b3a</v>
+        <v>f75f3579-4010-42c4-80e2-f2a7cfd71402</v>
       </c>
       <c r="B35" t="str">
-        <v>e323d9c8-295f-472c-93f3-fefc39655d80</v>
+        <v>4f0a6d51-f2bc-4517-bdbe-9b39a26ebb5d</v>
       </c>
       <c r="C35" t="str">
-        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
+        <v>55d6e756-c40c-4755-84ab-c3458437acd6</v>
       </c>
       <c r="D35" t="str">
         <v>0</v>
       </c>
       <c r="E35" t="str">
-        <v>2026-09-11T06:56:21.627Z</v>
+        <v>2026-09-11T08:18:25.620Z</v>
       </c>
       <c r="F35" t="str">
-        <v>2026-09-11T06:56:21.627Z</v>
+        <v>2026-09-11T08:18:25.620Z</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>96cc8b37-e673-419a-bf8d-08393ece27ae</v>
+        <v>36e49927-d354-4adc-af39-4c65b2974184</v>
       </c>
       <c r="B36" t="str">
-        <v>6ac09b86-b7ee-4b62-b048-4594eca71b6c</v>
+        <v>f503ee00-c9c6-4e8f-b72e-bc09d0fec90e</v>
       </c>
       <c r="C36" t="str">
+        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
+      </c>
+      <c r="D36" t="str">
+        <v>0</v>
+      </c>
+      <c r="E36" t="str">
+        <v>2026-09-11T08:22:00.406Z</v>
+      </c>
+      <c r="F36" t="str">
+        <v>2026-09-11T08:22:00.406Z</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>dc16ef5e-6f03-4f0a-8539-a1727bf6cf7e</v>
+      </c>
+      <c r="B37" t="str">
+        <v>f503ee00-c9c6-4e8f-b72e-bc09d0fec90e</v>
+      </c>
+      <c r="C37" t="str">
+        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
+      </c>
+      <c r="D37" t="str">
+        <v>1</v>
+      </c>
+      <c r="E37" t="str">
+        <v>2026-09-11T08:22:00.414Z</v>
+      </c>
+      <c r="F37" t="str">
+        <v>2026-09-11T08:22:00.414Z</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>ecb99d03-fb1d-45d2-b60d-4bc7c1affd0d</v>
+      </c>
+      <c r="B38" t="str">
+        <v>2702b682-23d0-4b69-a895-7bd6d6a3965f</v>
+      </c>
+      <c r="C38" t="str">
+        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
+      </c>
+      <c r="D38" t="str">
+        <v>0</v>
+      </c>
+      <c r="E38" t="str">
+        <v>2026-09-11T08:22:33.266Z</v>
+      </c>
+      <c r="F38" t="str">
+        <v>2026-09-11T08:22:33.266Z</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>038f1f4c-8f4d-4019-9161-59593c954b0a</v>
+      </c>
+      <c r="B39" t="str">
+        <v>a3bbee49-623f-4bc2-935b-a989adca81ca</v>
+      </c>
+      <c r="C39" t="str">
+        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
+      </c>
+      <c r="D39" t="str">
+        <v>0</v>
+      </c>
+      <c r="E39" t="str">
+        <v>2026-09-11T08:22:44.180Z</v>
+      </c>
+      <c r="F39" t="str">
+        <v>2026-09-11T08:22:44.180Z</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>f131ff6d-b891-4fc8-b9e6-9fb49b343f53</v>
+      </c>
+      <c r="B40" t="str">
+        <v>a3bbee49-623f-4bc2-935b-a989adca81ca</v>
+      </c>
+      <c r="C40" t="str">
+        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
+      </c>
+      <c r="D40" t="str">
+        <v>1</v>
+      </c>
+      <c r="E40" t="str">
+        <v>2026-09-11T08:22:44.190Z</v>
+      </c>
+      <c r="F40" t="str">
+        <v>2026-09-11T08:22:44.190Z</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>d958a365-d1c3-4ca6-80ad-c0db3ea7ac0b</v>
+      </c>
+      <c r="B41" t="str">
+        <v>c0a292e6-7ae6-4e30-a09f-b6551efd53a4</v>
+      </c>
+      <c r="C41" t="str">
+        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
+      </c>
+      <c r="D41" t="str">
+        <v>0</v>
+      </c>
+      <c r="E41" t="str">
+        <v>2026-09-11T08:23:10.518Z</v>
+      </c>
+      <c r="F41" t="str">
+        <v>2026-09-11T08:23:10.518Z</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>f72c8ce5-f9f2-4017-948d-839dd57380db</v>
+      </c>
+      <c r="B42" t="str">
+        <v>c0a292e6-7ae6-4e30-a09f-b6551efd53a4</v>
+      </c>
+      <c r="C42" t="str">
+        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
+      </c>
+      <c r="D42" t="str">
+        <v>1</v>
+      </c>
+      <c r="E42" t="str">
+        <v>2026-09-11T08:23:10.527Z</v>
+      </c>
+      <c r="F42" t="str">
+        <v>2026-09-11T08:23:10.527Z</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>ac6a9e88-c451-4e43-9953-4ce1b263280c</v>
+      </c>
+      <c r="B43" t="str">
+        <v>ada990db-b47a-4ec0-b8c6-03c068f69af6</v>
+      </c>
+      <c r="C43" t="str">
         <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
       </c>
-      <c r="D36" t="str">
-        <v>0</v>
-      </c>
-      <c r="E36" t="str">
-        <v>2026-09-11T06:58:59.731Z</v>
-      </c>
-      <c r="F36" t="str">
-        <v>2026-09-11T06:58:59.731Z</v>
+      <c r="D43" t="str">
+        <v>0</v>
+      </c>
+      <c r="E43" t="str">
+        <v>2026-09-11T08:23:27.684Z</v>
+      </c>
+      <c r="F43" t="str">
+        <v>2026-09-11T08:23:27.684Z</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>cec75ed0-f305-49f8-84e8-f2761dc66a7b</v>
+      </c>
+      <c r="B44" t="str">
+        <v>e323d9c8-295f-472c-93f3-fefc39655d80</v>
+      </c>
+      <c r="C44" t="str">
+        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
+      </c>
+      <c r="D44" t="str">
+        <v>0</v>
+      </c>
+      <c r="E44" t="str">
+        <v>2026-09-11T08:28:37.987Z</v>
+      </c>
+      <c r="F44" t="str">
+        <v>2026-09-11T08:28:37.987Z</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>92d67c64-2b4d-495a-abf5-4750262601d4</v>
+      </c>
+      <c r="B45" t="str">
+        <v>46019afc-2896-43ad-821c-552404768662</v>
+      </c>
+      <c r="C45" t="str">
+        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
+      </c>
+      <c r="D45" t="str">
+        <v>0</v>
+      </c>
+      <c r="E45" t="str">
+        <v>2026-09-11T08:34:52.092Z</v>
+      </c>
+      <c r="F45" t="str">
+        <v>2026-09-11T08:34:52.092Z</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>ba0e23ec-5cb4-4e82-b937-6175ffe77fb4</v>
+      </c>
+      <c r="B46" t="str">
+        <v>46019afc-2896-43ad-821c-552404768662</v>
+      </c>
+      <c r="C46" t="str">
+        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
+      </c>
+      <c r="D46" t="str">
+        <v>1</v>
+      </c>
+      <c r="E46" t="str">
+        <v>2026-09-11T08:34:52.102Z</v>
+      </c>
+      <c r="F46" t="str">
+        <v>2026-09-11T08:34:52.102Z</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>d8693219-b379-4848-abd8-26b275f5427c</v>
+      </c>
+      <c r="B47" t="str">
+        <v>576fbffe-152c-4052-834c-1d230af3784a</v>
+      </c>
+      <c r="C47" t="str">
+        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
+      </c>
+      <c r="D47" t="str">
+        <v>0</v>
+      </c>
+      <c r="E47" t="str">
+        <v>2026-09-11T08:41:43.787Z</v>
+      </c>
+      <c r="F47" t="str">
+        <v>2026-09-11T08:41:43.787Z</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>d8ab3b84-59c7-4d36-a813-fd2c9920f4bd</v>
+      </c>
+      <c r="B48" t="str">
+        <v>576fbffe-152c-4052-834c-1d230af3784a</v>
+      </c>
+      <c r="C48" t="str">
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+      </c>
+      <c r="D48" t="str">
+        <v>1</v>
+      </c>
+      <c r="E48" t="str">
+        <v>2026-09-11T08:41:43.796Z</v>
+      </c>
+      <c r="F48" t="str">
+        <v>2026-09-11T08:41:43.796Z</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>5f6ecf46-861f-4ddd-b97b-39359036e880</v>
+      </c>
+      <c r="B49" t="str">
+        <v>c1b2bc1d-f4c5-42ea-bdc8-4fdc41bfd8ee</v>
+      </c>
+      <c r="C49" t="str">
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+      </c>
+      <c r="D49" t="str">
+        <v>0</v>
+      </c>
+      <c r="E49" t="str">
+        <v>2026-09-11T08:42:08.145Z</v>
+      </c>
+      <c r="F49" t="str">
+        <v>2026-09-11T08:42:08.145Z</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>d3d148ca-b67b-4ed0-b7d0-78dcc2829541</v>
+      </c>
+      <c r="B50" t="str">
+        <v>a2d08247-d1c8-4c29-9663-96adb51418ff</v>
+      </c>
+      <c r="C50" t="str">
+        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
+      </c>
+      <c r="D50" t="str">
+        <v>0</v>
+      </c>
+      <c r="E50" t="str">
+        <v>2026-09-11T08:42:24.908Z</v>
+      </c>
+      <c r="F50" t="str">
+        <v>2026-09-11T08:42:24.908Z</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>b3e4f339-1eef-4005-b1ae-cc00c5188696</v>
+      </c>
+      <c r="B51" t="str">
+        <v>a2d08247-d1c8-4c29-9663-96adb51418ff</v>
+      </c>
+      <c r="C51" t="str">
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+      </c>
+      <c r="D51" t="str">
+        <v>1</v>
+      </c>
+      <c r="E51" t="str">
+        <v>2026-09-11T08:42:24.916Z</v>
+      </c>
+      <c r="F51" t="str">
+        <v>2026-09-11T08:42:24.916Z</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>a104ca08-2f34-4540-87b0-c78bcb4c9f24</v>
+      </c>
+      <c r="B52" t="str">
+        <v>4aef4aa0-8e8b-4280-b75a-f6df9d48e73a</v>
+      </c>
+      <c r="C52" t="str">
+        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
+      </c>
+      <c r="D52" t="str">
+        <v>0</v>
+      </c>
+      <c r="E52" t="str">
+        <v>2026-09-11T09:14:25.167Z</v>
+      </c>
+      <c r="F52" t="str">
+        <v>2026-09-11T09:14:25.167Z</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>c2574065-afba-483f-b672-a966d9af5fe7</v>
+      </c>
+      <c r="B53" t="str">
+        <v>4aef4aa0-8e8b-4280-b75a-f6df9d48e73a</v>
+      </c>
+      <c r="C53" t="str">
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+      </c>
+      <c r="D53" t="str">
+        <v>1</v>
+      </c>
+      <c r="E53" t="str">
+        <v>2026-09-11T09:14:25.174Z</v>
+      </c>
+      <c r="F53" t="str">
+        <v>2026-09-11T09:14:25.174Z</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>f027caa9-6164-4f17-9792-420177eda3ea</v>
+      </c>
+      <c r="B54" t="str">
+        <v>2033fe99-69ce-47d7-bed5-92a5d6bdedc3</v>
+      </c>
+      <c r="C54" t="str">
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+      </c>
+      <c r="D54" t="str">
+        <v>0</v>
+      </c>
+      <c r="E54" t="str">
+        <v>2026-09-11T09:14:33.039Z</v>
+      </c>
+      <c r="F54" t="str">
+        <v>2026-09-11T09:14:33.039Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F54"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>